<commit_message>
Add printer bid sheet with bid increase rules and suggested bids
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KT1VW3oarL8CCbJcMVGP8
</commit_message>
<xml_diff>
--- a/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
+++ b/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
@@ -7,19 +7,24 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입찰가 변경 전후" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="광고 기본 정보" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="키워드ID·링크" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프린터 입찰가" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입찰가 변경 전후" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="광고 기본 정보" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="키워드ID·링크" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'프린터 입찰가'!$A$13:$P$63</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0&quot;원&quot;"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +50,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF595959"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -73,8 +86,18 @@
         <fgColor rgb="FFFFE5E5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFE0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -96,11 +119,88 @@
         <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +227,53 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -493,6 +640,3105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>입찰가 인상 기준 (노란 칸 숫자를 바꾸면 추천 입찰가가 자동으로 다시 계산됩니다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>인상률</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>솔바텍 광고가 안 보임 → 노출되도록 크게 인상</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>솔바텍이 다른 사이트보다 2계단 이상 아래</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>붙어있음(아래)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>솔바텍이 다른 사이트 바로 아래 (예: 6위·5위)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>붙어있음(위)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>솔바텍이 바로 위지만 붙어 있음 (예: 1위·2위) → 간격 벌리기</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>순위 낮음</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>다른 사이트는 없지만 솔바텍 순위가 낮음</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>수정 대상 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>입찰가 상한</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>추천 입찰가는 이 금액을 넘지 않음 (10원 단위 올림). 현재 입찰가가 이미 상한보다 높으면 현재 금액 유지</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>※ 네이버 광고관리 &gt; 키워드 &gt; 입찰가 변경 &gt; "순위별 평균 입찰가"에서 목표 순위 금액을 확인해 L열에 넣으면 그 금액이 최종 입찰가가 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>키워드</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>광고업체수</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>솔바텍</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>코스모스몰</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>sb렌탈</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>입찰가 수정</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>현재 입찰가</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>인상률</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>추천 입찰가</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>네이버 목표순위 입찰가
+(직접 입력)</t>
+        </is>
+      </c>
+      <c r="M13" s="1" t="inlineStr">
+        <is>
+          <t>최종 변경 입찰가</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="inlineStr">
+        <is>
+          <t>노출수</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t>클릭수</t>
+        </is>
+      </c>
+      <c r="P13" s="1" t="inlineStr">
+        <is>
+          <t>평균 CPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>감열식프린터</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="J14" s="20">
+        <f>VLOOKUP(H14,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K14" s="19">
+        <f>IF(J14=0,I14,MAX(I14,MIN($B$10,ROUNDUP(I14*(1+J14),-1))))</f>
+        <v/>
+      </c>
+      <c r="L14" s="21" t="n"/>
+      <c r="M14" s="22">
+        <f>IF(L14&lt;&gt;"",MIN($B$10,L14),K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="18" t="n">
+        <v>23</v>
+      </c>
+      <c r="O14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>감열프린터</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J15" s="20">
+        <f>VLOOKUP(H15,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K15" s="19">
+        <f>IF(J15=0,I15,MAX(I15,MIN($B$10,ROUNDUP(I15*(1+J15),-1))))</f>
+        <v/>
+      </c>
+      <c r="L15" s="21" t="n"/>
+      <c r="M15" s="22">
+        <f>IF(L15&lt;&gt;"",MIN($B$10,L15),K15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="18" t="n">
+        <v>27</v>
+      </c>
+      <c r="O15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>감열프린터기</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="F16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="n">
+        <v>650</v>
+      </c>
+      <c r="J16" s="26">
+        <f>VLOOKUP(H16,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K16" s="25">
+        <f>IF(J16=0,I16,MAX(I16,MIN($B$10,ROUNDUP(I16*(1+J16),-1))))</f>
+        <v/>
+      </c>
+      <c r="L16" s="21" t="n"/>
+      <c r="M16" s="27">
+        <f>IF(L16&lt;&gt;"",MIN($B$10,L16),K16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="O16" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>도시바프린터</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J17" s="20">
+        <f>VLOOKUP(H17,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K17" s="19">
+        <f>IF(J17=0,I17,MAX(I17,MIN($B$10,ROUNDUP(I17*(1+J17),-1))))</f>
+        <v/>
+      </c>
+      <c r="L17" s="21" t="n"/>
+      <c r="M17" s="22">
+        <f>IF(L17&lt;&gt;"",MIN($B$10,L17),K17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="O17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>라밸프린터</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="23" t="n"/>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I18" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J18" s="26">
+        <f>VLOOKUP(H18,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K18" s="25">
+        <f>IF(J18=0,I18,MAX(I18,MIN($B$10,ROUNDUP(I18*(1+J18),-1))))</f>
+        <v/>
+      </c>
+      <c r="L18" s="21" t="n"/>
+      <c r="M18" s="27">
+        <f>IF(L18&lt;&gt;"",MIN($B$10,L18),K18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>라벨기</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
+      <c r="F19" s="23" t="n"/>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I19" s="25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J19" s="26">
+        <f>VLOOKUP(H19,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K19" s="25">
+        <f>IF(J19=0,I19,MAX(I19,MIN($B$10,ROUNDUP(I19*(1+J19),-1))))</f>
+        <v/>
+      </c>
+      <c r="L19" s="21" t="n"/>
+      <c r="M19" s="27">
+        <f>IF(L19&lt;&gt;"",MIN($B$10,L19),K19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>라벨기계</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="23" t="n"/>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I20" s="25" t="n">
+        <v>890</v>
+      </c>
+      <c r="J20" s="26">
+        <f>VLOOKUP(H20,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K20" s="25">
+        <f>IF(J20=0,I20,MAX(I20,MIN($B$10,ROUNDUP(I20*(1+J20),-1))))</f>
+        <v/>
+      </c>
+      <c r="L20" s="21" t="n"/>
+      <c r="M20" s="27">
+        <f>IF(L20&lt;&gt;"",MIN($B$10,L20),K20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>라벨용지프린터</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="23" t="n"/>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I21" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J21" s="26">
+        <f>VLOOKUP(H21,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K21" s="25">
+        <f>IF(J21=0,I21,MAX(I21,MIN($B$10,ROUNDUP(I21*(1+J21),-1))))</f>
+        <v/>
+      </c>
+      <c r="L21" s="21" t="n"/>
+      <c r="M21" s="27">
+        <f>IF(L21&lt;&gt;"",MIN($B$10,L21),K21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I22" s="25" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J22" s="26">
+        <f>VLOOKUP(H22,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K22" s="25">
+        <f>IF(J22=0,I22,MAX(I22,MIN($B$10,ROUNDUP(I22*(1+J22),-1))))</f>
+        <v/>
+      </c>
+      <c r="L22" s="21" t="n"/>
+      <c r="M22" s="27">
+        <f>IF(L22&lt;&gt;"",MIN($B$10,L22),K22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>라벨인쇄기계</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I23" s="25" t="n">
+        <v>600</v>
+      </c>
+      <c r="J23" s="26">
+        <f>VLOOKUP(H23,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K23" s="25">
+        <f>IF(J23=0,I23,MAX(I23,MIN($B$10,ROUNDUP(I23*(1+J23),-1))))</f>
+        <v/>
+      </c>
+      <c r="L23" s="21" t="n"/>
+      <c r="M23" s="27">
+        <f>IF(L23&lt;&gt;"",MIN($B$10,L23),K23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>라벨지프린터</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="23" t="n"/>
+      <c r="G24" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="n">
+        <v>800</v>
+      </c>
+      <c r="J24" s="26">
+        <f>VLOOKUP(H24,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K24" s="25">
+        <f>IF(J24=0,I24,MAX(I24,MIN($B$10,ROUNDUP(I24*(1+J24),-1))))</f>
+        <v/>
+      </c>
+      <c r="L24" s="21" t="n"/>
+      <c r="M24" s="27">
+        <f>IF(L24&lt;&gt;"",MIN($B$10,L24),K24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="O24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>라벨출력기</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I25" s="25" t="n">
+        <v>1110</v>
+      </c>
+      <c r="J25" s="26">
+        <f>VLOOKUP(H25,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K25" s="25">
+        <f>IF(J25=0,I25,MAX(I25,MIN($B$10,ROUNDUP(I25*(1+J25),-1))))</f>
+        <v/>
+      </c>
+      <c r="L25" s="21" t="n"/>
+      <c r="M25" s="27">
+        <f>IF(L25&lt;&gt;"",MIN($B$10,L25),K25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>라벨프린터업체</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H26" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="n">
+        <v>530</v>
+      </c>
+      <c r="J26" s="26">
+        <f>VLOOKUP(H26,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K26" s="25">
+        <f>IF(J26=0,I26,MAX(I26,MIN($B$10,ROUNDUP(I26*(1+J26),-1))))</f>
+        <v/>
+      </c>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="27">
+        <f>IF(L26&lt;&gt;"",MIN($B$10,L26),K26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>라벨프린터추천</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>붙어있음(위)</t>
+        </is>
+      </c>
+      <c r="I27" s="25" t="n">
+        <v>1580</v>
+      </c>
+      <c r="J27" s="26">
+        <f>VLOOKUP(H27,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K27" s="25">
+        <f>IF(J27=0,I27,MAX(I27,MIN($B$10,ROUNDUP(I27*(1+J27),-1))))</f>
+        <v/>
+      </c>
+      <c r="L27" s="21" t="n"/>
+      <c r="M27" s="27">
+        <f>IF(L27&lt;&gt;"",MIN($B$10,L27),K27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>롤라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="23" t="n"/>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="J28" s="26">
+        <f>VLOOKUP(H28,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K28" s="25">
+        <f>IF(J28=0,I28,MAX(I28,MIN($B$10,ROUNDUP(I28*(1+J28),-1))))</f>
+        <v/>
+      </c>
+      <c r="L28" s="21" t="n"/>
+      <c r="M28" s="27">
+        <f>IF(L28&lt;&gt;"",MIN($B$10,L28),K28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>롤라벨출력기</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" s="23" t="n"/>
+      <c r="E29" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="23" t="n"/>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" s="26">
+        <f>VLOOKUP(H29,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K29" s="25">
+        <f>IF(J29=0,I29,MAX(I29,MIN($B$10,ROUNDUP(I29*(1+J29),-1))))</f>
+        <v/>
+      </c>
+      <c r="L29" s="21" t="n"/>
+      <c r="M29" s="27">
+        <f>IF(L29&lt;&gt;"",MIN($B$10,L29),K29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>롤라벨프린터</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="23" t="n"/>
+      <c r="F30" s="23" t="n"/>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H30" s="23" t="inlineStr">
+        <is>
+          <t>순위 낮음</t>
+        </is>
+      </c>
+      <c r="I30" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J30" s="26">
+        <f>VLOOKUP(H30,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K30" s="25">
+        <f>IF(J30=0,I30,MAX(I30,MIN($B$10,ROUNDUP(I30*(1+J30),-1))))</f>
+        <v/>
+      </c>
+      <c r="L30" s="21" t="n"/>
+      <c r="M30" s="27">
+        <f>IF(L30&lt;&gt;"",MIN($B$10,L30),K30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>바코드라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="23" t="n"/>
+      <c r="G31" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I31" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="J31" s="26">
+        <f>VLOOKUP(H31,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K31" s="25">
+        <f>IF(J31=0,I31,MAX(I31,MIN($B$10,ROUNDUP(I31*(1+J31),-1))))</f>
+        <v/>
+      </c>
+      <c r="L31" s="21" t="n"/>
+      <c r="M31" s="27">
+        <f>IF(L31&lt;&gt;"",MIN($B$10,L31),K31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>바코드라벨프린터</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="23" t="n"/>
+      <c r="G32" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I32" s="25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J32" s="26">
+        <f>VLOOKUP(H32,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K32" s="25">
+        <f>IF(J32=0,I32,MAX(I32,MIN($B$10,ROUNDUP(I32*(1+J32),-1))))</f>
+        <v/>
+      </c>
+      <c r="L32" s="21" t="n"/>
+      <c r="M32" s="27">
+        <f>IF(L32&lt;&gt;"",MIN($B$10,L32),K32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="O32" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="23" t="inlineStr">
+        <is>
+          <t>3,100원</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>바코드라벨프린터업체</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="23" t="n"/>
+      <c r="G33" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I33" s="25" t="n">
+        <v>300</v>
+      </c>
+      <c r="J33" s="26">
+        <f>VLOOKUP(H33,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K33" s="25">
+        <f>IF(J33=0,I33,MAX(I33,MIN($B$10,ROUNDUP(I33*(1+J33),-1))))</f>
+        <v/>
+      </c>
+      <c r="L33" s="21" t="n"/>
+      <c r="M33" s="27">
+        <f>IF(L33&lt;&gt;"",MIN($B$10,L33),K33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>바코드만들기</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>중지: 키워드 OFF</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" s="23" t="n"/>
+      <c r="E34" s="23" t="n"/>
+      <c r="F34" s="23" t="n"/>
+      <c r="G34" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I34" s="25" t="n">
+        <v>500</v>
+      </c>
+      <c r="J34" s="26">
+        <f>VLOOKUP(H34,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K34" s="25">
+        <f>IF(J34=0,I34,MAX(I34,MIN($B$10,ROUNDUP(I34*(1+J34),-1))))</f>
+        <v/>
+      </c>
+      <c r="L34" s="21" t="n"/>
+      <c r="M34" s="27">
+        <f>IF(L34&lt;&gt;"",MIN($B$10,L34),K34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>바코드발행기</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" s="23" t="n"/>
+      <c r="E35" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I35" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="J35" s="26">
+        <f>VLOOKUP(H35,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K35" s="25">
+        <f>IF(J35=0,I35,MAX(I35,MIN($B$10,ROUNDUP(I35*(1+J35),-1))))</f>
+        <v/>
+      </c>
+      <c r="L35" s="21" t="n"/>
+      <c r="M35" s="27">
+        <f>IF(L35&lt;&gt;"",MIN($B$10,L35),K35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>바코드인쇄기</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" s="23" t="n"/>
+      <c r="E36" s="23" t="n"/>
+      <c r="F36" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I36" s="25" t="n">
+        <v>3300</v>
+      </c>
+      <c r="J36" s="26">
+        <f>VLOOKUP(H36,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K36" s="25">
+        <f>IF(J36=0,I36,MAX(I36,MIN($B$10,ROUNDUP(I36*(1+J36),-1))))</f>
+        <v/>
+      </c>
+      <c r="L36" s="21" t="n"/>
+      <c r="M36" s="27">
+        <f>IF(L36&lt;&gt;"",MIN($B$10,L36),K36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="O36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>바코드출력기</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I37" s="25" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J37" s="26">
+        <f>VLOOKUP(H37,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K37" s="25">
+        <f>IF(J37=0,I37,MAX(I37,MIN($B$10,ROUNDUP(I37*(1+J37),-1))))</f>
+        <v/>
+      </c>
+      <c r="L37" s="21" t="n"/>
+      <c r="M37" s="27">
+        <f>IF(L37&lt;&gt;"",MIN($B$10,L37),K37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="O37" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터기</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="23" t="n"/>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I38" s="25" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J38" s="26">
+        <f>VLOOKUP(H38,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K38" s="25">
+        <f>IF(J38=0,I38,MAX(I38,MIN($B$10,ROUNDUP(I38*(1+J38),-1))))</f>
+        <v/>
+      </c>
+      <c r="L38" s="21" t="n"/>
+      <c r="M38" s="27">
+        <f>IF(L38&lt;&gt;"",MIN($B$10,L38),K38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터라벨</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E39" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="23" t="n"/>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I39" s="25" t="n">
+        <v>1100</v>
+      </c>
+      <c r="J39" s="26">
+        <f>VLOOKUP(H39,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K39" s="25">
+        <f>IF(J39=0,I39,MAX(I39,MIN($B$10,ROUNDUP(I39*(1+J39),-1))))</f>
+        <v/>
+      </c>
+      <c r="L39" s="21" t="n"/>
+      <c r="M39" s="27">
+        <f>IF(L39&lt;&gt;"",MIN($B$10,L39),K39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터전문업체</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="23" t="n"/>
+      <c r="E40" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="23" t="n"/>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I40" s="25" t="n">
+        <v>700</v>
+      </c>
+      <c r="J40" s="26">
+        <f>VLOOKUP(H40,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K40" s="25">
+        <f>IF(J40=0,I40,MAX(I40,MIN($B$10,ROUNDUP(I40*(1+J40),-1))))</f>
+        <v/>
+      </c>
+      <c r="L40" s="21" t="n"/>
+      <c r="M40" s="27">
+        <f>IF(L40&lt;&gt;"",MIN($B$10,L40),K40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터추천</t>
+        </is>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D41" s="23" t="n"/>
+      <c r="E41" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="F41" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H41" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I41" s="25" t="n">
+        <v>1700</v>
+      </c>
+      <c r="J41" s="26">
+        <f>VLOOKUP(H41,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K41" s="25">
+        <f>IF(J41=0,I41,MAX(I41,MIN($B$10,ROUNDUP(I41*(1+J41),-1))))</f>
+        <v/>
+      </c>
+      <c r="L41" s="21" t="n"/>
+      <c r="M41" s="27">
+        <f>IF(L41&lt;&gt;"",MIN($B$10,L41),K41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터판매</t>
+        </is>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="23" t="n"/>
+      <c r="E42" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="23" t="n"/>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H42" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I42" s="25" t="n">
+        <v>280</v>
+      </c>
+      <c r="J42" s="26">
+        <f>VLOOKUP(H42,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K42" s="25">
+        <f>IF(J42=0,I42,MAX(I42,MIN($B$10,ROUNDUP(I42*(1+J42),-1))))</f>
+        <v/>
+      </c>
+      <c r="L42" s="21" t="n"/>
+      <c r="M42" s="27">
+        <f>IF(L42&lt;&gt;"",MIN($B$10,L42),K42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>바코드프린터프로그램</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C43" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="18" t="n"/>
+      <c r="H43" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I43" s="19" t="n">
+        <v>2750</v>
+      </c>
+      <c r="J43" s="20">
+        <f>VLOOKUP(H43,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K43" s="19">
+        <f>IF(J43=0,I43,MAX(I43,MIN($B$10,ROUNDUP(I43*(1+J43),-1))))</f>
+        <v/>
+      </c>
+      <c r="L43" s="21" t="n"/>
+      <c r="M43" s="22">
+        <f>IF(L43&lt;&gt;"",MIN($B$10,L43),K43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>빅솔론</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D44" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="18" t="n"/>
+      <c r="F44" s="18" t="n"/>
+      <c r="G44" s="18" t="n"/>
+      <c r="H44" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I44" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="J44" s="20">
+        <f>VLOOKUP(H44,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K44" s="19">
+        <f>IF(J44=0,I44,MAX(I44,MIN($B$10,ROUNDUP(I44*(1+J44),-1))))</f>
+        <v/>
+      </c>
+      <c r="L44" s="21" t="n"/>
+      <c r="M44" s="22">
+        <f>IF(L44&lt;&gt;"",MIN($B$10,L44),K44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="18" t="n">
+        <v>562</v>
+      </c>
+      <c r="O44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>빅솔론총판</t>
+        </is>
+      </c>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" s="23" t="n"/>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I45" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="J45" s="26">
+        <f>VLOOKUP(H45,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K45" s="25">
+        <f>IF(J45=0,I45,MAX(I45,MIN($B$10,ROUNDUP(I45*(1+J45),-1))))</f>
+        <v/>
+      </c>
+      <c r="L45" s="21" t="n"/>
+      <c r="M45" s="27">
+        <f>IF(L45&lt;&gt;"",MIN($B$10,L45),K45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>빅솔론프린터</t>
+        </is>
+      </c>
+      <c r="B46" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E46" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H46" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I46" s="25" t="n">
+        <v>940</v>
+      </c>
+      <c r="J46" s="26">
+        <f>VLOOKUP(H46,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K46" s="25">
+        <f>IF(J46=0,I46,MAX(I46,MIN($B$10,ROUNDUP(I46*(1+J46),-1))))</f>
+        <v/>
+      </c>
+      <c r="L46" s="21" t="n"/>
+      <c r="M46" s="27">
+        <f>IF(L46&lt;&gt;"",MIN($B$10,L46),K46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="23" t="n">
+        <v>43</v>
+      </c>
+      <c r="O46" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>산업용라벨프린터</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E47" s="18" t="n"/>
+      <c r="F47" s="18" t="n"/>
+      <c r="G47" s="18" t="n"/>
+      <c r="H47" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J47" s="20">
+        <f>VLOOKUP(H47,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K47" s="19">
+        <f>IF(J47=0,I47,MAX(I47,MIN($B$10,ROUNDUP(I47*(1+J47),-1))))</f>
+        <v/>
+      </c>
+      <c r="L47" s="21" t="n"/>
+      <c r="M47" s="22">
+        <f>IF(L47&lt;&gt;"",MIN($B$10,L47),K47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="O47" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P47" s="18" t="inlineStr">
+        <is>
+          <t>4,970원</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>산업용바코드프린터</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="23" t="n"/>
+      <c r="E48" s="23" t="n"/>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H48" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I48" s="25" t="n">
+        <v>800</v>
+      </c>
+      <c r="J48" s="26">
+        <f>VLOOKUP(H48,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K48" s="25">
+        <f>IF(J48=0,I48,MAX(I48,MIN($B$10,ROUNDUP(I48*(1+J48),-1))))</f>
+        <v/>
+      </c>
+      <c r="L48" s="21" t="n"/>
+      <c r="M48" s="27">
+        <f>IF(L48&lt;&gt;"",MIN($B$10,L48),K48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>산업용프린터</t>
+        </is>
+      </c>
+      <c r="B49" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D49" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H49" s="23" t="inlineStr">
+        <is>
+          <t>붙어있음(위)</t>
+        </is>
+      </c>
+      <c r="I49" s="25" t="n">
+        <v>6500</v>
+      </c>
+      <c r="J49" s="26">
+        <f>VLOOKUP(H49,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K49" s="25">
+        <f>IF(J49=0,I49,MAX(I49,MIN($B$10,ROUNDUP(I49*(1+J49),-1))))</f>
+        <v/>
+      </c>
+      <c r="L49" s="21" t="n"/>
+      <c r="M49" s="27">
+        <f>IF(L49&lt;&gt;"",MIN($B$10,L49),K49)</f>
+        <v/>
+      </c>
+      <c r="N49" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="O49" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P49" s="23" t="inlineStr">
+        <is>
+          <t>6,578원</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>소형바코드프린터</t>
+        </is>
+      </c>
+      <c r="B50" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D50" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E50" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H50" s="23" t="inlineStr">
+        <is>
+          <t>붙어있음(아래)</t>
+        </is>
+      </c>
+      <c r="I50" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J50" s="26">
+        <f>VLOOKUP(H50,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K50" s="25">
+        <f>IF(J50=0,I50,MAX(I50,MIN($B$10,ROUNDUP(I50*(1+J50),-1))))</f>
+        <v/>
+      </c>
+      <c r="L50" s="21" t="n"/>
+      <c r="M50" s="27">
+        <f>IF(L50&lt;&gt;"",MIN($B$10,L50),K50)</f>
+        <v/>
+      </c>
+      <c r="N50" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>스티커라벨기</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C51" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" s="23" t="n"/>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H51" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I51" s="25" t="n">
+        <v>2300</v>
+      </c>
+      <c r="J51" s="26">
+        <f>VLOOKUP(H51,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K51" s="25">
+        <f>IF(J51=0,I51,MAX(I51,MIN($B$10,ROUNDUP(I51*(1+J51),-1))))</f>
+        <v/>
+      </c>
+      <c r="L51" s="21" t="n"/>
+      <c r="M51" s="27">
+        <f>IF(L51&lt;&gt;"",MIN($B$10,L51),K51)</f>
+        <v/>
+      </c>
+      <c r="N51" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="O51" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>스티커인쇄기</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="18" t="n"/>
+      <c r="E52" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="18" t="n"/>
+      <c r="H52" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I52" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="J52" s="20">
+        <f>VLOOKUP(H52,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K52" s="19">
+        <f>IF(J52=0,I52,MAX(I52,MIN($B$10,ROUNDUP(I52*(1+J52),-1))))</f>
+        <v/>
+      </c>
+      <c r="L52" s="21" t="n"/>
+      <c r="M52" s="22">
+        <f>IF(L52&lt;&gt;"",MIN($B$10,L52),K52)</f>
+        <v/>
+      </c>
+      <c r="N52" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="O52" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>스티커출력기</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C53" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D53" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H53" s="23" t="inlineStr">
+        <is>
+          <t>순위 차이 큼</t>
+        </is>
+      </c>
+      <c r="I53" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="J53" s="26">
+        <f>VLOOKUP(H53,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K53" s="25">
+        <f>IF(J53=0,I53,MAX(I53,MIN($B$10,ROUNDUP(I53*(1+J53),-1))))</f>
+        <v/>
+      </c>
+      <c r="L53" s="21" t="n"/>
+      <c r="M53" s="27">
+        <f>IF(L53&lt;&gt;"",MIN($B$10,L53),K53)</f>
+        <v/>
+      </c>
+      <c r="N53" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="O53" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>스티커프린터</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D54" s="23" t="n"/>
+      <c r="E54" s="23" t="n"/>
+      <c r="F54" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H54" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I54" s="25" t="n">
+        <v>1340</v>
+      </c>
+      <c r="J54" s="26">
+        <f>VLOOKUP(H54,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K54" s="25">
+        <f>IF(J54=0,I54,MAX(I54,MIN($B$10,ROUNDUP(I54*(1+J54),-1))))</f>
+        <v/>
+      </c>
+      <c r="L54" s="21" t="n"/>
+      <c r="M54" s="27">
+        <f>IF(L54&lt;&gt;"",MIN($B$10,L54),K54)</f>
+        <v/>
+      </c>
+      <c r="N54" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O54" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>열전사프린터</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="D55" s="23" t="n"/>
+      <c r="E55" s="23" t="n"/>
+      <c r="F55" s="23" t="n"/>
+      <c r="G55" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H55" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I55" s="25" t="n">
+        <v>5500</v>
+      </c>
+      <c r="J55" s="26">
+        <f>VLOOKUP(H55,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K55" s="25">
+        <f>IF(J55=0,I55,MAX(I55,MIN($B$10,ROUNDUP(I55*(1+J55),-1))))</f>
+        <v/>
+      </c>
+      <c r="L55" s="21" t="n"/>
+      <c r="M55" s="27">
+        <f>IF(L55&lt;&gt;"",MIN($B$10,L55),K55)</f>
+        <v/>
+      </c>
+      <c r="N55" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="O55" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>열전사프린터기</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D56" s="23" t="n"/>
+      <c r="E56" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="F56" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G56" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H56" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I56" s="25" t="n">
+        <v>450</v>
+      </c>
+      <c r="J56" s="26">
+        <f>VLOOKUP(H56,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K56" s="25">
+        <f>IF(J56=0,I56,MAX(I56,MIN($B$10,ROUNDUP(I56*(1+J56),-1))))</f>
+        <v/>
+      </c>
+      <c r="L56" s="21" t="n"/>
+      <c r="M56" s="27">
+        <f>IF(L56&lt;&gt;"",MIN($B$10,L56),K56)</f>
+        <v/>
+      </c>
+      <c r="N56" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>영수증프린터</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E57" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="23" t="n"/>
+      <c r="G57" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H57" s="23" t="inlineStr">
+        <is>
+          <t>붙어있음(위)</t>
+        </is>
+      </c>
+      <c r="I57" s="25" t="n">
+        <v>1070</v>
+      </c>
+      <c r="J57" s="26">
+        <f>VLOOKUP(H57,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K57" s="25">
+        <f>IF(J57=0,I57,MAX(I57,MIN($B$10,ROUNDUP(I57*(1+J57),-1))))</f>
+        <v/>
+      </c>
+      <c r="L57" s="21" t="n"/>
+      <c r="M57" s="27">
+        <f>IF(L57&lt;&gt;"",MIN($B$10,L57),K57)</f>
+        <v/>
+      </c>
+      <c r="N57" s="23" t="n">
+        <v>85</v>
+      </c>
+      <c r="O57" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>제브라</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E58" s="18" t="n"/>
+      <c r="F58" s="18" t="n"/>
+      <c r="G58" s="18" t="n"/>
+      <c r="H58" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I58" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J58" s="20">
+        <f>VLOOKUP(H58,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K58" s="19">
+        <f>IF(J58=0,I58,MAX(I58,MIN($B$10,ROUNDUP(I58*(1+J58),-1))))</f>
+        <v/>
+      </c>
+      <c r="L58" s="21" t="n"/>
+      <c r="M58" s="22">
+        <f>IF(L58&lt;&gt;"",MIN($B$10,L58),K58)</f>
+        <v/>
+      </c>
+      <c r="N58" s="18" t="n">
+        <v>115</v>
+      </c>
+      <c r="O58" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" s="18" t="inlineStr">
+        <is>
+          <t>1,464원</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>제브라라벨프린터</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D59" s="23" t="n"/>
+      <c r="E59" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F59" s="23" t="n"/>
+      <c r="G59" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H59" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I59" s="25" t="n">
+        <v>700</v>
+      </c>
+      <c r="J59" s="26">
+        <f>VLOOKUP(H59,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K59" s="25">
+        <f>IF(J59=0,I59,MAX(I59,MIN($B$10,ROUNDUP(I59*(1+J59),-1))))</f>
+        <v/>
+      </c>
+      <c r="L59" s="21" t="n"/>
+      <c r="M59" s="27">
+        <f>IF(L59&lt;&gt;"",MIN($B$10,L59),K59)</f>
+        <v/>
+      </c>
+      <c r="N59" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="O59" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>제브라바코드프린터</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D60" s="23" t="n"/>
+      <c r="E60" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="F60" s="23" t="n"/>
+      <c r="G60" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H60" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J60" s="26">
+        <f>VLOOKUP(H60,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K60" s="25">
+        <f>IF(J60=0,I60,MAX(I60,MIN($B$10,ROUNDUP(I60*(1+J60),-1))))</f>
+        <v/>
+      </c>
+      <c r="L60" s="21" t="n"/>
+      <c r="M60" s="27">
+        <f>IF(L60&lt;&gt;"",MIN($B$10,L60),K60)</f>
+        <v/>
+      </c>
+      <c r="N60" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O60" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>제브라프린터</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>노출가능</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D61" s="23" t="n"/>
+      <c r="E61" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F61" s="23" t="n"/>
+      <c r="G61" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H61" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I61" s="25" t="n">
+        <v>1410</v>
+      </c>
+      <c r="J61" s="26">
+        <f>VLOOKUP(H61,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K61" s="25">
+        <f>IF(J61=0,I61,MAX(I61,MIN($B$10,ROUNDUP(I61*(1+J61),-1))))</f>
+        <v/>
+      </c>
+      <c r="L61" s="21" t="n"/>
+      <c r="M61" s="27">
+        <f>IF(L61&lt;&gt;"",MIN($B$10,L61),K61)</f>
+        <v/>
+      </c>
+      <c r="N61" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O61" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>카드프린터기</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>중지: 키워드 OFF</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" s="23" t="n"/>
+      <c r="E62" s="23" t="n"/>
+      <c r="F62" s="23" t="n"/>
+      <c r="G62" s="24" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="H62" s="23" t="inlineStr">
+        <is>
+          <t>솔바텍 미노출</t>
+        </is>
+      </c>
+      <c r="I62" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="J62" s="26">
+        <f>VLOOKUP(H62,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K62" s="25">
+        <f>IF(J62=0,I62,MAX(I62,MIN($B$10,ROUNDUP(I62*(1+J62),-1))))</f>
+        <v/>
+      </c>
+      <c r="L62" s="21" t="n"/>
+      <c r="M62" s="27">
+        <f>IF(L62&lt;&gt;"",MIN($B$10,L62),K62)</f>
+        <v/>
+      </c>
+      <c r="N62" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" s="23" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>프린터관리</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>중지: 키워드 OFF</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="18" t="n"/>
+      <c r="F63" s="18" t="n"/>
+      <c r="G63" s="18" t="n"/>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>유지</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="J63" s="20">
+        <f>VLOOKUP(H63,$A$3:$B$8,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="K63" s="19">
+        <f>IF(J63=0,I63,MAX(I63,MIN($B$10,ROUNDUP(I63*(1+J63),-1))))</f>
+        <v/>
+      </c>
+      <c r="L63" s="21" t="n"/>
+      <c r="M63" s="22">
+        <f>IF(L63&lt;&gt;"",MIN($B$10,L63),K63)</f>
+        <v/>
+      </c>
+      <c r="N63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" s="18" t="inlineStr">
+        <is>
+          <t>0원</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A13:P63"/>
+  <mergeCells count="8">
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C2:F2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H14:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=$A$3:$A$8</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -521,22 +3767,23 @@
           <t>입찰가 변경 전</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
+      <c r="C1" s="28" t="n"/>
+      <c r="D1" s="28" t="n"/>
+      <c r="E1" s="28" t="n"/>
+      <c r="F1" s="28" t="n"/>
+      <c r="G1" s="29" t="n"/>
       <c r="H1" s="4" t="inlineStr">
         <is>
           <t>입찰가 변경 후</t>
         </is>
       </c>
-      <c r="I1" s="5" t="n"/>
-      <c r="J1" s="5" t="n"/>
-      <c r="K1" s="5" t="n"/>
-      <c r="L1" s="5" t="n"/>
+      <c r="I1" s="28" t="n"/>
+      <c r="J1" s="28" t="n"/>
+      <c r="K1" s="28" t="n"/>
+      <c r="L1" s="29" t="n"/>
     </row>
     <row r="2">
+      <c r="A2" s="30" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>현재 입찰가</t>
@@ -6059,7 +9306,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H305" s="9" t="n"/>
+      <c r="H305" s="31">
+        <f>'프린터 입찰가'!M21</f>
+        <v/>
+      </c>
       <c r="I305" s="9" t="n"/>
       <c r="J305" s="9" t="n"/>
       <c r="K305" s="9" t="n"/>
@@ -6087,7 +9337,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H306" s="9" t="n"/>
+      <c r="H306" s="31">
+        <f>'프린터 입찰가'!M23</f>
+        <v/>
+      </c>
       <c r="I306" s="9" t="n"/>
       <c r="J306" s="9" t="n"/>
       <c r="K306" s="9" t="n"/>
@@ -6115,7 +9368,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H307" s="9" t="n"/>
+      <c r="H307" s="31">
+        <f>'프린터 입찰가'!M24</f>
+        <v/>
+      </c>
       <c r="I307" s="9" t="n"/>
       <c r="J307" s="9" t="n"/>
       <c r="K307" s="9" t="n"/>
@@ -6143,7 +9399,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H308" s="9" t="n"/>
+      <c r="H308" s="31">
+        <f>'프린터 입찰가'!M26</f>
+        <v/>
+      </c>
       <c r="I308" s="9" t="n"/>
       <c r="J308" s="9" t="n"/>
       <c r="K308" s="9" t="n"/>
@@ -6173,7 +9432,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H309" s="9" t="n"/>
+      <c r="H309" s="31">
+        <f>'프린터 입찰가'!M27</f>
+        <v/>
+      </c>
       <c r="I309" s="9" t="n"/>
       <c r="J309" s="9" t="n"/>
       <c r="K309" s="9" t="n"/>
@@ -6201,7 +9463,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H310" s="9" t="n"/>
+      <c r="H310" s="31">
+        <f>'프린터 입찰가'!M31</f>
+        <v/>
+      </c>
       <c r="I310" s="9" t="n"/>
       <c r="J310" s="9" t="n"/>
       <c r="K310" s="9" t="n"/>
@@ -6229,7 +9494,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H311" s="9" t="n"/>
+      <c r="H311" s="31">
+        <f>'프린터 입찰가'!M36</f>
+        <v/>
+      </c>
       <c r="I311" s="9" t="n"/>
       <c r="J311" s="9" t="n"/>
       <c r="K311" s="9" t="n"/>
@@ -6259,7 +9527,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H312" s="9" t="n"/>
+      <c r="H312" s="31">
+        <f>'프린터 입찰가'!M41</f>
+        <v/>
+      </c>
       <c r="I312" s="9" t="n"/>
       <c r="J312" s="9" t="n"/>
       <c r="K312" s="9" t="n"/>
@@ -6311,7 +9582,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H314" s="9" t="n"/>
+      <c r="H314" s="31">
+        <f>'프린터 입찰가'!M59</f>
+        <v/>
+      </c>
       <c r="I314" s="9" t="n"/>
       <c r="J314" s="9" t="n"/>
       <c r="K314" s="9" t="n"/>
@@ -6339,7 +9613,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H315" s="9" t="n"/>
+      <c r="H315" s="31">
+        <f>'프린터 입찰가'!M60</f>
+        <v/>
+      </c>
       <c r="I315" s="9" t="n"/>
       <c r="J315" s="9" t="n"/>
       <c r="K315" s="9" t="n"/>
@@ -6367,7 +9644,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H316" s="9" t="n"/>
+      <c r="H316" s="31">
+        <f>'프린터 입찰가'!M33</f>
+        <v/>
+      </c>
       <c r="I316" s="9" t="n"/>
       <c r="J316" s="9" t="n"/>
       <c r="K316" s="9" t="n"/>
@@ -6395,7 +9675,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H317" s="9" t="n"/>
+      <c r="H317" s="31">
+        <f>'프린터 입찰가'!M40</f>
+        <v/>
+      </c>
       <c r="I317" s="9" t="n"/>
       <c r="J317" s="9" t="n"/>
       <c r="K317" s="9" t="n"/>
@@ -6469,7 +9752,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H320" s="9" t="n"/>
+      <c r="H320" s="31">
+        <f>'프린터 입찰가'!M20</f>
+        <v/>
+      </c>
       <c r="I320" s="9" t="n"/>
       <c r="J320" s="9" t="n"/>
       <c r="K320" s="9" t="n"/>
@@ -6497,7 +9783,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H321" s="9" t="n"/>
+      <c r="H321" s="31">
+        <f>'프린터 입찰가'!M35</f>
+        <v/>
+      </c>
       <c r="I321" s="9" t="n"/>
       <c r="J321" s="9" t="n"/>
       <c r="K321" s="9" t="n"/>
@@ -6525,7 +9814,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H322" s="9" t="n"/>
+      <c r="H322" s="31">
+        <f>'프린터 입찰가'!M42</f>
+        <v/>
+      </c>
       <c r="I322" s="9" t="n"/>
       <c r="J322" s="9" t="n"/>
       <c r="K322" s="9" t="n"/>
@@ -6555,7 +9847,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H323" s="9" t="n"/>
+      <c r="H323" s="31">
+        <f>'프린터 입찰가'!M46</f>
+        <v/>
+      </c>
       <c r="I323" s="9" t="n"/>
       <c r="J323" s="9" t="n"/>
       <c r="K323" s="9" t="n"/>
@@ -6585,7 +9880,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H324" s="9" t="n"/>
+      <c r="H324" s="31">
+        <f>'프린터 입찰가'!M50</f>
+        <v/>
+      </c>
       <c r="I324" s="9" t="n"/>
       <c r="J324" s="9" t="n"/>
       <c r="K324" s="9" t="n"/>
@@ -6637,7 +9935,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H326" s="9" t="n"/>
+      <c r="H326" s="31">
+        <f>'프린터 입찰가'!M61</f>
+        <v/>
+      </c>
       <c r="I326" s="9" t="n"/>
       <c r="J326" s="9" t="n"/>
       <c r="K326" s="9" t="n"/>
@@ -6687,7 +9988,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H328" s="9" t="n"/>
+      <c r="H328" s="31">
+        <f>'프린터 입찰가'!M45</f>
+        <v/>
+      </c>
       <c r="I328" s="9" t="n"/>
       <c r="J328" s="9" t="n"/>
       <c r="K328" s="9" t="n"/>
@@ -6713,7 +10017,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H329" s="9" t="n"/>
+      <c r="H329" s="31">
+        <f>'프린터 입찰가'!M48</f>
+        <v/>
+      </c>
       <c r="I329" s="9" t="n"/>
       <c r="J329" s="9" t="n"/>
       <c r="K329" s="9" t="n"/>
@@ -6743,7 +10050,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H330" s="9" t="n"/>
+      <c r="H330" s="31">
+        <f>'프린터 입찰가'!M49</f>
+        <v/>
+      </c>
       <c r="I330" s="9" t="n"/>
       <c r="J330" s="9" t="n"/>
       <c r="K330" s="9" t="n"/>
@@ -6769,7 +10079,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H331" s="9" t="n"/>
+      <c r="H331" s="31">
+        <f>'프린터 입찰가'!M51</f>
+        <v/>
+      </c>
       <c r="I331" s="9" t="n"/>
       <c r="J331" s="9" t="n"/>
       <c r="K331" s="9" t="n"/>
@@ -6797,7 +10110,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H332" s="9" t="n"/>
+      <c r="H332" s="31">
+        <f>'프린터 입찰가'!M54</f>
+        <v/>
+      </c>
       <c r="I332" s="9" t="n"/>
       <c r="J332" s="9" t="n"/>
       <c r="K332" s="9" t="n"/>
@@ -6853,7 +10169,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H334" s="9" t="n"/>
+      <c r="H334" s="31">
+        <f>'프린터 입찰가'!M53</f>
+        <v/>
+      </c>
       <c r="I334" s="9" t="n"/>
       <c r="J334" s="9" t="n"/>
       <c r="K334" s="9" t="n"/>
@@ -6881,7 +10200,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H335" s="9" t="n"/>
+      <c r="H335" s="31">
+        <f>'프린터 입찰가'!M30</f>
+        <v/>
+      </c>
       <c r="I335" s="9" t="n"/>
       <c r="J335" s="9" t="n"/>
       <c r="K335" s="9" t="n"/>
@@ -6909,7 +10231,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H336" s="9" t="n"/>
+      <c r="H336" s="31">
+        <f>'프린터 입찰가'!M29</f>
+        <v/>
+      </c>
       <c r="I336" s="9" t="n"/>
       <c r="J336" s="9" t="n"/>
       <c r="K336" s="9" t="n"/>
@@ -6937,7 +10262,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H337" s="9" t="n"/>
+      <c r="H337" s="31">
+        <f>'프린터 입찰가'!M28</f>
+        <v/>
+      </c>
       <c r="I337" s="9" t="n"/>
       <c r="J337" s="9" t="n"/>
       <c r="K337" s="9" t="n"/>
@@ -6967,7 +10295,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H338" s="9" t="n"/>
+      <c r="H338" s="31">
+        <f>'프린터 입찰가'!M57</f>
+        <v/>
+      </c>
       <c r="I338" s="9" t="n"/>
       <c r="J338" s="9" t="n"/>
       <c r="K338" s="9" t="n"/>
@@ -6999,7 +10330,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H339" s="9" t="n"/>
+      <c r="H339" s="31">
+        <f>'프린터 입찰가'!M16</f>
+        <v/>
+      </c>
       <c r="I339" s="9" t="n"/>
       <c r="J339" s="9" t="n"/>
       <c r="K339" s="9" t="n"/>
@@ -7029,7 +10363,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H340" s="9" t="n"/>
+      <c r="H340" s="31">
+        <f>'프린터 입찰가'!M56</f>
+        <v/>
+      </c>
       <c r="I340" s="9" t="n"/>
       <c r="J340" s="9" t="n"/>
       <c r="K340" s="9" t="n"/>
@@ -7055,7 +10392,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H341" s="9" t="n"/>
+      <c r="H341" s="31">
+        <f>'프린터 입찰가'!M55</f>
+        <v/>
+      </c>
       <c r="I341" s="9" t="n"/>
       <c r="J341" s="9" t="n"/>
       <c r="K341" s="9" t="n"/>
@@ -7107,7 +10447,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H343" s="9" t="n"/>
+      <c r="H343" s="31">
+        <f>'프린터 입찰가'!M19</f>
+        <v/>
+      </c>
       <c r="I343" s="9" t="n"/>
       <c r="J343" s="9" t="n"/>
       <c r="K343" s="9" t="n"/>
@@ -7139,7 +10482,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H344" s="9" t="n"/>
+      <c r="H344" s="31">
+        <f>'프린터 입찰가'!M37</f>
+        <v/>
+      </c>
       <c r="I344" s="9" t="n"/>
       <c r="J344" s="9" t="n"/>
       <c r="K344" s="9" t="n"/>
@@ -7169,7 +10515,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H345" s="9" t="n"/>
+      <c r="H345" s="31">
+        <f>'프린터 입찰가'!M25</f>
+        <v/>
+      </c>
       <c r="I345" s="9" t="n"/>
       <c r="J345" s="9" t="n"/>
       <c r="K345" s="9" t="n"/>
@@ -7199,7 +10548,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H346" s="9" t="n"/>
+      <c r="H346" s="31">
+        <f>'프린터 입찰가'!M39</f>
+        <v/>
+      </c>
       <c r="I346" s="9" t="n"/>
       <c r="J346" s="9" t="n"/>
       <c r="K346" s="9" t="n"/>
@@ -7227,7 +10579,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H347" s="9" t="n"/>
+      <c r="H347" s="31">
+        <f>'프린터 입찰가'!M18</f>
+        <v/>
+      </c>
       <c r="I347" s="9" t="n"/>
       <c r="J347" s="9" t="n"/>
       <c r="K347" s="9" t="n"/>
@@ -7255,7 +10610,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H348" s="9" t="n"/>
+      <c r="H348" s="31">
+        <f>'프린터 입찰가'!M38</f>
+        <v/>
+      </c>
       <c r="I348" s="9" t="n"/>
       <c r="J348" s="9" t="n"/>
       <c r="K348" s="9" t="n"/>
@@ -7285,7 +10643,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H349" s="9" t="n"/>
+      <c r="H349" s="31">
+        <f>'프린터 입찰가'!M32</f>
+        <v/>
+      </c>
       <c r="I349" s="9" t="n"/>
       <c r="J349" s="9" t="n"/>
       <c r="K349" s="9" t="n"/>
@@ -7313,7 +10674,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H350" s="9" t="n"/>
+      <c r="H350" s="31">
+        <f>'프린터 입찰가'!M22</f>
+        <v/>
+      </c>
       <c r="I350" s="9" t="n"/>
       <c r="J350" s="9" t="n"/>
       <c r="K350" s="9" t="n"/>
@@ -8761,7 +12125,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H430" s="9" t="n"/>
+      <c r="H430" s="31">
+        <f>'프린터 입찰가'!M34</f>
+        <v/>
+      </c>
       <c r="I430" s="9" t="n"/>
       <c r="J430" s="9" t="n"/>
       <c r="K430" s="9" t="n"/>
@@ -8787,7 +12154,10 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H431" s="9" t="n"/>
+      <c r="H431" s="31">
+        <f>'프린터 입찰가'!M62</f>
+        <v/>
+      </c>
       <c r="I431" s="9" t="n"/>
       <c r="J431" s="9" t="n"/>
       <c r="K431" s="9" t="n"/>
@@ -8825,7 +12195,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17783,7 +21153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Replace printer bid sheet with per-site bid and rank comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KT1VW3oarL8CCbJcMVGP8
</commit_message>
<xml_diff>
--- a/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
+++ b/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="키워드ID·링크" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'프린터 입찰가'!$A$13:$P$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'프린터 입찰가'!$A$2:$I$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,10 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0&quot;원&quot;"/>
-  </numFmts>
-  <fonts count="7">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,16 +48,8 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF595959"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -84,16 +74,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE5E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFE0"/>
       </patternFill>
     </fill>
   </fills>
@@ -200,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -228,53 +208,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -640,3095 +591,1324 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P63"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
-          <t>입찰가 인상 기준 (노란 칸 숫자를 바꾸면 추천 입찰가가 자동으로 다시 계산됩니다)</t>
-        </is>
-      </c>
+          <t>키워드</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>입찰가 수정</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>광고업체수</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>입찰가</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>노출순위</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="5" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>판정</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>인상률</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>설명</t>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>솔바텍</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>코스모스몰</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>sb렌탈</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>솔바텍</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>코스모스몰</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>sb렌탈</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>솔바텍 광고가 안 보임 → 노출되도록 크게 인상</t>
-        </is>
-      </c>
+          <t>감열식프린터</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="E3" s="16" t="n"/>
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>솔바텍이 다른 사이트보다 2계단 이상 아래</t>
-        </is>
+          <t>감열프린터</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="16" t="n"/>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>붙어있음(아래)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>솔바텍이 다른 사이트 바로 아래 (예: 6위·5위)</t>
-        </is>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>감열프린터기</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>650</v>
+      </c>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>붙어있음(위)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>솔바텍이 바로 위지만 붙어 있음 (예: 1위·2위) → 간격 벌리기</t>
-        </is>
-      </c>
+          <t>도시바프린터</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>순위 낮음</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>다른 사이트는 없지만 솔바텍 순위가 낮음</t>
-        </is>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>라밸프린터</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>수정 대상 아님</t>
-        </is>
-      </c>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>라벨기</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>라벨기계</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>890</v>
+      </c>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>입찰가 상한</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>추천 입찰가는 이 금액을 넘지 않음 (10원 단위 올림). 현재 입찰가가 이미 상한보다 높으면 현재 금액 유지</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>라벨용지프린터</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="9" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>※ 네이버 광고관리 &gt; 키워드 &gt; 입찰가 변경 &gt; "순위별 평균 입찰가"에서 목표 순위 금액을 확인해 L열에 넣으면 그 금액이 최종 입찰가가 됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>키워드</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>상태</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>광고업체수</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>솔바텍</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>코스모스몰</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>sb렌탈</t>
-        </is>
-      </c>
-      <c r="G13" s="1" t="inlineStr">
-        <is>
-          <t>입찰가 수정</t>
-        </is>
-      </c>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>판정</t>
-        </is>
-      </c>
-      <c r="I13" s="1" t="inlineStr">
-        <is>
-          <t>현재 입찰가</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="inlineStr">
-        <is>
-          <t>인상률</t>
-        </is>
-      </c>
-      <c r="K13" s="1" t="inlineStr">
-        <is>
-          <t>추천 입찰가</t>
-        </is>
-      </c>
-      <c r="L13" s="17" t="inlineStr">
-        <is>
-          <t>네이버 목표순위 입찰가
-(직접 입력)</t>
-        </is>
-      </c>
-      <c r="M13" s="1" t="inlineStr">
-        <is>
-          <t>최종 변경 입찰가</t>
-        </is>
-      </c>
-      <c r="N13" s="1" t="inlineStr">
-        <is>
-          <t>노출수</t>
-        </is>
-      </c>
-      <c r="O13" s="1" t="inlineStr">
-        <is>
-          <t>클릭수</t>
-        </is>
-      </c>
-      <c r="P13" s="1" t="inlineStr">
-        <is>
-          <t>평균 CPC</t>
-        </is>
-      </c>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>라벨인쇄기계</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>600</v>
+      </c>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>라벨지프린터</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>800</v>
+      </c>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="9" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>감열식프린터</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="n">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>라벨출력기</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D14" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I14" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="J14" s="20">
-        <f>VLOOKUP(H14,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K14" s="19">
-        <f>IF(J14=0,I14,MAX(I14,MIN($B$10,ROUNDUP(I14*(1+J14),-1))))</f>
-        <v/>
-      </c>
-      <c r="L14" s="21" t="n"/>
-      <c r="M14" s="22">
-        <f>IF(L14&lt;&gt;"",MIN($B$10,L14),K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="18" t="n">
-        <v>23</v>
-      </c>
-      <c r="O14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D14" s="17" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>감열프린터</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="n">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>라벨프린터업체</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D15" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n">
+      <c r="D15" s="17" t="n">
+        <v>530</v>
+      </c>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J15" s="20">
-        <f>VLOOKUP(H15,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K15" s="19">
-        <f>IF(J15=0,I15,MAX(I15,MIN($B$10,ROUNDUP(I15*(1+J15),-1))))</f>
-        <v/>
-      </c>
-      <c r="L15" s="21" t="n"/>
-      <c r="M15" s="22">
-        <f>IF(L15&lt;&gt;"",MIN($B$10,L15),K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="O15" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="I15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>감열프린터기</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="n">
+          <t>라벨프린터추천</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" s="23" t="n">
+      <c r="D16" s="17" t="n">
+        <v>1580</v>
+      </c>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="F16" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="24" t="inlineStr">
+      <c r="H16" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>롤라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H16" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I16" s="25" t="n">
-        <v>650</v>
-      </c>
-      <c r="J16" s="26">
-        <f>VLOOKUP(H16,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K16" s="25">
-        <f>IF(J16=0,I16,MAX(I16,MIN($B$10,ROUNDUP(I16*(1+J16),-1))))</f>
-        <v/>
-      </c>
-      <c r="L16" s="21" t="n"/>
-      <c r="M16" s="27">
-        <f>IF(L16&lt;&gt;"",MIN($B$10,L16),K16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="O16" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>도시바프린터</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D17" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J17" s="20">
-        <f>VLOOKUP(H17,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K17" s="19">
-        <f>IF(J17=0,I17,MAX(I17,MIN($B$10,ROUNDUP(I17*(1+J17),-1))))</f>
-        <v/>
-      </c>
-      <c r="L17" s="21" t="n"/>
-      <c r="M17" s="22">
-        <f>IF(L17&lt;&gt;"",MIN($B$10,L17),K17)</f>
-        <v/>
-      </c>
-      <c r="N17" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D17" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>라밸프린터</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" s="23" t="n"/>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="24" t="inlineStr">
+          <t>롤라벨출력기</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H18" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I18" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J18" s="26">
-        <f>VLOOKUP(H18,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K18" s="25">
-        <f>IF(J18=0,I18,MAX(I18,MIN($B$10,ROUNDUP(I18*(1+J18),-1))))</f>
-        <v/>
-      </c>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="27">
-        <f>IF(L18&lt;&gt;"",MIN($B$10,L18),K18)</f>
-        <v/>
-      </c>
-      <c r="N18" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>라벨기</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n">
+          <t>롤라벨프린터</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H19" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I19" s="25" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J19" s="26">
-        <f>VLOOKUP(H19,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K19" s="25">
-        <f>IF(J19=0,I19,MAX(I19,MIN($B$10,ROUNDUP(I19*(1+J19),-1))))</f>
-        <v/>
-      </c>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="27">
-        <f>IF(L19&lt;&gt;"",MIN($B$10,L19),K19)</f>
-        <v/>
-      </c>
-      <c r="N19" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="O19" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D19" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>라벨기계</t>
-        </is>
-      </c>
-      <c r="B20" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="n">
+          <t>바코드라벨인쇄기</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="23" t="n"/>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="23" t="n"/>
-      <c r="G20" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I20" s="25" t="n">
-        <v>890</v>
-      </c>
-      <c r="J20" s="26">
-        <f>VLOOKUP(H20,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K20" s="25">
-        <f>IF(J20=0,I20,MAX(I20,MIN($B$10,ROUNDUP(I20*(1+J20),-1))))</f>
-        <v/>
-      </c>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="27">
-        <f>IF(L20&lt;&gt;"",MIN($B$10,L20),K20)</f>
-        <v/>
-      </c>
-      <c r="N20" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D20" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>라벨용지프린터</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" s="23" t="n"/>
-      <c r="E21" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" s="23" t="n"/>
-      <c r="G21" s="24" t="inlineStr">
+          <t>바코드라벨프린터</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H21" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I21" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J21" s="26">
-        <f>VLOOKUP(H21,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K21" s="25">
-        <f>IF(J21=0,I21,MAX(I21,MIN($B$10,ROUNDUP(I21*(1+J21),-1))))</f>
-        <v/>
-      </c>
-      <c r="L21" s="21" t="n"/>
-      <c r="M21" s="27">
-        <f>IF(L21&lt;&gt;"",MIN($B$10,L21),K21)</f>
-        <v/>
-      </c>
-      <c r="N21" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C21" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" s="17" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D22" s="23" t="n"/>
-      <c r="E22" s="23" t="n"/>
-      <c r="F22" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="24" t="inlineStr">
+          <t>바코드라벨프린터업체</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H22" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I22" s="25" t="n">
-        <v>3500</v>
-      </c>
-      <c r="J22" s="26">
-        <f>VLOOKUP(H22,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K22" s="25">
-        <f>IF(J22=0,I22,MAX(I22,MIN($B$10,ROUNDUP(I22*(1+J22),-1))))</f>
-        <v/>
-      </c>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="27">
-        <f>IF(L22&lt;&gt;"",MIN($B$10,L22),K22)</f>
-        <v/>
-      </c>
-      <c r="N22" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="O22" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C22" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기계</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C23" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D23" s="23" t="n"/>
-      <c r="E23" s="23" t="n"/>
-      <c r="F23" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" s="24" t="inlineStr">
+          <t>바코드만들기</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H23" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I23" s="25" t="n">
-        <v>600</v>
-      </c>
-      <c r="J23" s="26">
-        <f>VLOOKUP(H23,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K23" s="25">
-        <f>IF(J23=0,I23,MAX(I23,MIN($B$10,ROUNDUP(I23*(1+J23),-1))))</f>
-        <v/>
-      </c>
-      <c r="L23" s="21" t="n"/>
-      <c r="M23" s="27">
-        <f>IF(L23&lt;&gt;"",MIN($B$10,L23),K23)</f>
-        <v/>
-      </c>
-      <c r="N23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C23" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>라벨지프린터</t>
-        </is>
-      </c>
-      <c r="B24" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C24" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D24" s="23" t="n"/>
-      <c r="E24" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="23" t="n"/>
-      <c r="G24" s="24" t="inlineStr">
+          <t>바코드발행기</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H24" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I24" s="25" t="n">
-        <v>800</v>
-      </c>
-      <c r="J24" s="26">
-        <f>VLOOKUP(H24,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K24" s="25">
-        <f>IF(J24=0,I24,MAX(I24,MIN($B$10,ROUNDUP(I24*(1+J24),-1))))</f>
-        <v/>
-      </c>
-      <c r="L24" s="21" t="n"/>
-      <c r="M24" s="27">
-        <f>IF(L24&lt;&gt;"",MIN($B$10,L24),K24)</f>
-        <v/>
-      </c>
-      <c r="N24" s="23" t="n">
+      <c r="C24" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="O24" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D24" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>라벨출력기</t>
-        </is>
-      </c>
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C25" s="23" t="n">
+          <t>바코드인쇄기</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D25" s="23" t="n">
+      <c r="D25" s="17" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+      <c r="I25" s="9" t="n">
         <v>7</v>
-      </c>
-      <c r="E25" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="23" t="n"/>
-      <c r="G25" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I25" s="25" t="n">
-        <v>1110</v>
-      </c>
-      <c r="J25" s="26">
-        <f>VLOOKUP(H25,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K25" s="25">
-        <f>IF(J25=0,I25,MAX(I25,MIN($B$10,ROUNDUP(I25*(1+J25),-1))))</f>
-        <v/>
-      </c>
-      <c r="L25" s="21" t="n"/>
-      <c r="M25" s="27">
-        <f>IF(L25&lt;&gt;"",MIN($B$10,L25),K25)</f>
-        <v/>
-      </c>
-      <c r="N25" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터업체</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C26" s="23" t="n">
+          <t>바코드출력기</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D26" s="23" t="n"/>
-      <c r="E26" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I26" s="25" t="n">
-        <v>530</v>
-      </c>
-      <c r="J26" s="26">
-        <f>VLOOKUP(H26,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K26" s="25">
-        <f>IF(J26=0,I26,MAX(I26,MIN($B$10,ROUNDUP(I26*(1+J26),-1))))</f>
-        <v/>
-      </c>
-      <c r="L26" s="21" t="n"/>
-      <c r="M26" s="27">
-        <f>IF(L26&lt;&gt;"",MIN($B$10,L26),K26)</f>
-        <v/>
-      </c>
-      <c r="N26" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
+      <c r="D26" s="17" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터추천</t>
-        </is>
-      </c>
-      <c r="B27" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D27" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="E27" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="F27" s="23" t="n"/>
-      <c r="G27" s="24" t="inlineStr">
+          <t>바코드프린터기</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H27" s="23" t="inlineStr">
-        <is>
-          <t>붙어있음(위)</t>
-        </is>
-      </c>
-      <c r="I27" s="25" t="n">
-        <v>1580</v>
-      </c>
-      <c r="J27" s="26">
-        <f>VLOOKUP(H27,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K27" s="25">
-        <f>IF(J27=0,I27,MAX(I27,MIN($B$10,ROUNDUP(I27*(1+J27),-1))))</f>
-        <v/>
-      </c>
-      <c r="L27" s="21" t="n"/>
-      <c r="M27" s="27">
-        <f>IF(L27&lt;&gt;"",MIN($B$10,L27),K27)</f>
-        <v/>
-      </c>
-      <c r="N27" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="O27" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C27" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>롤라벨인쇄기</t>
-        </is>
-      </c>
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D28" s="23" t="n"/>
-      <c r="E28" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="23" t="n"/>
-      <c r="G28" s="24" t="inlineStr">
+          <t>바코드프린터라벨</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H28" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I28" s="25" t="n">
-        <v>70</v>
-      </c>
-      <c r="J28" s="26">
-        <f>VLOOKUP(H28,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K28" s="25">
-        <f>IF(J28=0,I28,MAX(I28,MIN($B$10,ROUNDUP(I28*(1+J28),-1))))</f>
-        <v/>
-      </c>
-      <c r="L28" s="21" t="n"/>
-      <c r="M28" s="27">
-        <f>IF(L28&lt;&gt;"",MIN($B$10,L28),K28)</f>
-        <v/>
-      </c>
-      <c r="N28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C28" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>롤라벨출력기</t>
-        </is>
-      </c>
-      <c r="B29" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C29" s="23" t="n">
+          <t>바코드프린터전문업체</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="23" t="n"/>
-      <c r="E29" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H29" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I29" s="25" t="n">
-        <v>100</v>
-      </c>
-      <c r="J29" s="26">
-        <f>VLOOKUP(H29,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K29" s="25">
-        <f>IF(J29=0,I29,MAX(I29,MIN($B$10,ROUNDUP(I29*(1+J29),-1))))</f>
-        <v/>
-      </c>
-      <c r="L29" s="21" t="n"/>
-      <c r="M29" s="27">
-        <f>IF(L29&lt;&gt;"",MIN($B$10,L29),K29)</f>
-        <v/>
-      </c>
-      <c r="N29" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D29" s="17" t="n">
+        <v>700</v>
+      </c>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>롤라벨프린터</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D30" s="23" t="n">
+          <t>바코드프린터추천</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E30" s="23" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>순위 낮음</t>
-        </is>
-      </c>
-      <c r="I30" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J30" s="26">
-        <f>VLOOKUP(H30,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K30" s="25">
-        <f>IF(J30=0,I30,MAX(I30,MIN($B$10,ROUNDUP(I30*(1+J30),-1))))</f>
-        <v/>
-      </c>
-      <c r="L30" s="21" t="n"/>
-      <c r="M30" s="27">
-        <f>IF(L30&lt;&gt;"",MIN($B$10,L30),K30)</f>
-        <v/>
-      </c>
-      <c r="N30" s="23" t="n">
+      <c r="D30" s="17" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I30" s="9" t="n">
         <v>1</v>
-      </c>
-      <c r="O30" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨인쇄기</t>
-        </is>
-      </c>
-      <c r="B31" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D31" s="23" t="n"/>
-      <c r="E31" s="23" t="n">
+          <t>바코드프린터판매</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H31" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I31" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="J31" s="26">
-        <f>VLOOKUP(H31,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K31" s="25">
-        <f>IF(J31=0,I31,MAX(I31,MIN($B$10,ROUNDUP(I31*(1+J31),-1))))</f>
-        <v/>
-      </c>
-      <c r="L31" s="21" t="n"/>
-      <c r="M31" s="27">
-        <f>IF(L31&lt;&gt;"",MIN($B$10,L31),K31)</f>
-        <v/>
-      </c>
-      <c r="N31" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D31" s="17" t="n">
+        <v>280</v>
+      </c>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>바코드라벨프린터</t>
-        </is>
-      </c>
-      <c r="B32" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C32" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D32" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="E32" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I32" s="25" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J32" s="26">
-        <f>VLOOKUP(H32,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K32" s="25">
-        <f>IF(J32=0,I32,MAX(I32,MIN($B$10,ROUNDUP(I32*(1+J32),-1))))</f>
-        <v/>
-      </c>
-      <c r="L32" s="21" t="n"/>
-      <c r="M32" s="27">
-        <f>IF(L32&lt;&gt;"",MIN($B$10,L32),K32)</f>
-        <v/>
-      </c>
-      <c r="N32" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="O32" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" s="23" t="inlineStr">
-        <is>
-          <t>3,100원</t>
-        </is>
-      </c>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>바코드프린터프로그램</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" s="16" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>바코드라벨프린터업체</t>
-        </is>
-      </c>
-      <c r="B33" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="n">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>빅솔론</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="23" t="n"/>
-      <c r="E33" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F33" s="23" t="n"/>
-      <c r="G33" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H33" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I33" s="25" t="n">
-        <v>300</v>
-      </c>
-      <c r="J33" s="26">
-        <f>VLOOKUP(H33,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K33" s="25">
-        <f>IF(J33=0,I33,MAX(I33,MIN($B$10,ROUNDUP(I33*(1+J33),-1))))</f>
-        <v/>
-      </c>
-      <c r="L33" s="21" t="n"/>
-      <c r="M33" s="27">
-        <f>IF(L33&lt;&gt;"",MIN($B$10,L33),K33)</f>
-        <v/>
-      </c>
-      <c r="N33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>바코드만들기</t>
-        </is>
-      </c>
-      <c r="B34" s="23" t="inlineStr">
-        <is>
-          <t>중지: 키워드 OFF</t>
-        </is>
-      </c>
-      <c r="C34" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="24" t="inlineStr">
+          <t>빅솔론총판</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H34" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I34" s="25" t="n">
-        <v>500</v>
-      </c>
-      <c r="J34" s="26">
-        <f>VLOOKUP(H34,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K34" s="25">
-        <f>IF(J34=0,I34,MAX(I34,MIN($B$10,ROUNDUP(I34*(1+J34),-1))))</f>
-        <v/>
-      </c>
-      <c r="L34" s="21" t="n"/>
-      <c r="M34" s="27">
-        <f>IF(L34&lt;&gt;"",MIN($B$10,L34),K34)</f>
-        <v/>
-      </c>
-      <c r="N34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C34" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>바코드발행기</t>
-        </is>
-      </c>
-      <c r="B35" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C35" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="24" t="inlineStr">
+          <t>빅솔론프린터</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H35" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I35" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="J35" s="26">
-        <f>VLOOKUP(H35,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K35" s="25">
-        <f>IF(J35=0,I35,MAX(I35,MIN($B$10,ROUNDUP(I35*(1+J35),-1))))</f>
-        <v/>
-      </c>
-      <c r="L35" s="21" t="n"/>
-      <c r="M35" s="27">
-        <f>IF(L35&lt;&gt;"",MIN($B$10,L35),K35)</f>
-        <v/>
-      </c>
-      <c r="N35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C35" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="17" t="n">
+        <v>940</v>
+      </c>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="9" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>바코드인쇄기</t>
-        </is>
-      </c>
-      <c r="B36" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C36" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G36" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H36" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I36" s="25" t="n">
-        <v>3300</v>
-      </c>
-      <c r="J36" s="26">
-        <f>VLOOKUP(H36,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K36" s="25">
-        <f>IF(J36=0,I36,MAX(I36,MIN($B$10,ROUNDUP(I36*(1+J36),-1))))</f>
-        <v/>
-      </c>
-      <c r="L36" s="21" t="n"/>
-      <c r="M36" s="27">
-        <f>IF(L36&lt;&gt;"",MIN($B$10,L36),K36)</f>
-        <v/>
-      </c>
-      <c r="N36" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="O36" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>산업용라벨프린터</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D36" s="16" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>바코드출력기</t>
-        </is>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C37" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D37" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="E37" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="F37" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="24" t="inlineStr">
+          <t>산업용바코드프린터</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H37" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I37" s="25" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J37" s="26">
-        <f>VLOOKUP(H37,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K37" s="25">
-        <f>IF(J37=0,I37,MAX(I37,MIN($B$10,ROUNDUP(I37*(1+J37),-1))))</f>
-        <v/>
-      </c>
-      <c r="L37" s="21" t="n"/>
-      <c r="M37" s="27">
-        <f>IF(L37&lt;&gt;"",MIN($B$10,L37),K37)</f>
-        <v/>
-      </c>
-      <c r="N37" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="O37" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C37" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <v>800</v>
+      </c>
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터기</t>
-        </is>
-      </c>
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C38" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D38" s="23" t="n"/>
-      <c r="E38" s="23" t="n">
+          <t>산업용프린터</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H38" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I38" s="25" t="n">
-        <v>4000</v>
-      </c>
-      <c r="J38" s="26">
-        <f>VLOOKUP(H38,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K38" s="25">
-        <f>IF(J38=0,I38,MAX(I38,MIN($B$10,ROUNDUP(I38*(1+J38),-1))))</f>
-        <v/>
-      </c>
-      <c r="L38" s="21" t="n"/>
-      <c r="M38" s="27">
-        <f>IF(L38&lt;&gt;"",MIN($B$10,L38),K38)</f>
-        <v/>
-      </c>
-      <c r="N38" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="O38" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="H38" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터라벨</t>
-        </is>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C39" s="23" t="n">
+          <t>소형바코드프린터</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D39" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="E39" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H39" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I39" s="25" t="n">
-        <v>1100</v>
-      </c>
-      <c r="J39" s="26">
-        <f>VLOOKUP(H39,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K39" s="25">
-        <f>IF(J39=0,I39,MAX(I39,MIN($B$10,ROUNDUP(I39*(1+J39),-1))))</f>
-        <v/>
-      </c>
-      <c r="L39" s="21" t="n"/>
-      <c r="M39" s="27">
-        <f>IF(L39&lt;&gt;"",MIN($B$10,L39),K39)</f>
-        <v/>
-      </c>
-      <c r="N39" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O39" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D39" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터전문업체</t>
-        </is>
-      </c>
-      <c r="B40" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C40" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D40" s="23" t="n"/>
-      <c r="E40" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="24" t="inlineStr">
+          <t>스티커라벨기</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H40" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I40" s="25" t="n">
-        <v>700</v>
-      </c>
-      <c r="J40" s="26">
-        <f>VLOOKUP(H40,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K40" s="25">
-        <f>IF(J40=0,I40,MAX(I40,MIN($B$10,ROUNDUP(I40*(1+J40),-1))))</f>
-        <v/>
-      </c>
-      <c r="L40" s="21" t="n"/>
-      <c r="M40" s="27">
-        <f>IF(L40&lt;&gt;"",MIN($B$10,L40),K40)</f>
-        <v/>
-      </c>
-      <c r="N40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C40" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>바코드프린터추천</t>
-        </is>
-      </c>
-      <c r="B41" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C41" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="D41" s="23" t="n"/>
-      <c r="E41" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="F41" s="23" t="n">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>스티커인쇄기</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="E41" s="16" t="n"/>
+      <c r="F41" s="16" t="n"/>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I41" s="7" t="n">
         <v>1</v>
-      </c>
-      <c r="G41" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H41" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I41" s="25" t="n">
-        <v>1700</v>
-      </c>
-      <c r="J41" s="26">
-        <f>VLOOKUP(H41,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K41" s="25">
-        <f>IF(J41=0,I41,MAX(I41,MIN($B$10,ROUNDUP(I41*(1+J41),-1))))</f>
-        <v/>
-      </c>
-      <c r="L41" s="21" t="n"/>
-      <c r="M41" s="27">
-        <f>IF(L41&lt;&gt;"",MIN($B$10,L41),K41)</f>
-        <v/>
-      </c>
-      <c r="N41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터판매</t>
-        </is>
-      </c>
-      <c r="B42" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C42" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D42" s="23" t="n"/>
-      <c r="E42" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" s="23" t="n"/>
-      <c r="G42" s="24" t="inlineStr">
+          <t>스티커출력기</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H42" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I42" s="25" t="n">
-        <v>280</v>
-      </c>
-      <c r="J42" s="26">
-        <f>VLOOKUP(H42,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K42" s="25">
-        <f>IF(J42=0,I42,MAX(I42,MIN($B$10,ROUNDUP(I42*(1+J42),-1))))</f>
-        <v/>
-      </c>
-      <c r="L42" s="21" t="n"/>
-      <c r="M42" s="27">
-        <f>IF(L42&lt;&gt;"",MIN($B$10,L42),K42)</f>
-        <v/>
-      </c>
-      <c r="N42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C42" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="E42" s="17" t="n"/>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>바코드프린터프로그램</t>
-        </is>
-      </c>
-      <c r="B43" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C43" s="18" t="n">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>스티커프린터</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <v>1340</v>
+      </c>
+      <c r="E43" s="17" t="n"/>
+      <c r="F43" s="17" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
+      <c r="I43" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>열전사프린터</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D43" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18" t="n"/>
-      <c r="H43" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I43" s="19" t="n">
-        <v>2750</v>
-      </c>
-      <c r="J43" s="20">
-        <f>VLOOKUP(H43,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K43" s="19">
-        <f>IF(J43=0,I43,MAX(I43,MIN($B$10,ROUNDUP(I43*(1+J43),-1))))</f>
-        <v/>
-      </c>
-      <c r="L43" s="21" t="n"/>
-      <c r="M43" s="22">
-        <f>IF(L43&lt;&gt;"",MIN($B$10,L43),K43)</f>
-        <v/>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="O43" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>빅솔론</t>
-        </is>
-      </c>
-      <c r="B44" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C44" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="D44" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="18" t="n"/>
-      <c r="H44" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I44" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="J44" s="20">
-        <f>VLOOKUP(H44,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K44" s="19">
-        <f>IF(J44=0,I44,MAX(I44,MIN($B$10,ROUNDUP(I44*(1+J44),-1))))</f>
-        <v/>
-      </c>
-      <c r="L44" s="21" t="n"/>
-      <c r="M44" s="22">
-        <f>IF(L44&lt;&gt;"",MIN($B$10,L44),K44)</f>
-        <v/>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>562</v>
-      </c>
-      <c r="O44" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D44" s="17" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E44" s="17" t="n"/>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
+      <c r="I44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>빅솔론총판</t>
-        </is>
-      </c>
-      <c r="B45" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C45" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="D45" s="23" t="n"/>
-      <c r="E45" s="23" t="n"/>
-      <c r="F45" s="23" t="n"/>
-      <c r="G45" s="24" t="inlineStr">
+          <t>열전사프린터기</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H45" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I45" s="25" t="n">
-        <v>70</v>
-      </c>
-      <c r="J45" s="26">
-        <f>VLOOKUP(H45,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K45" s="25">
-        <f>IF(J45=0,I45,MAX(I45,MIN($B$10,ROUNDUP(I45*(1+J45),-1))))</f>
-        <v/>
-      </c>
-      <c r="L45" s="21" t="n"/>
-      <c r="M45" s="27">
-        <f>IF(L45&lt;&gt;"",MIN($B$10,L45),K45)</f>
-        <v/>
-      </c>
-      <c r="N45" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O45" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
+      <c r="C45" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="17" t="n">
+        <v>450</v>
+      </c>
+      <c r="E45" s="17" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I45" s="9" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>빅솔론프린터</t>
-        </is>
-      </c>
-      <c r="B46" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C46" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D46" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="E46" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="23" t="n"/>
-      <c r="G46" s="24" t="inlineStr">
+          <t>영수증프린터</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H46" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I46" s="25" t="n">
-        <v>940</v>
-      </c>
-      <c r="J46" s="26">
-        <f>VLOOKUP(H46,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K46" s="25">
-        <f>IF(J46=0,I46,MAX(I46,MIN($B$10,ROUNDUP(I46*(1+J46),-1))))</f>
-        <v/>
-      </c>
-      <c r="L46" s="21" t="n"/>
-      <c r="M46" s="27">
-        <f>IF(L46&lt;&gt;"",MIN($B$10,L46),K46)</f>
-        <v/>
-      </c>
-      <c r="N46" s="23" t="n">
-        <v>43</v>
-      </c>
-      <c r="O46" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P46" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C46" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D46" s="17" t="n">
+        <v>1070</v>
+      </c>
+      <c r="E46" s="17" t="n"/>
+      <c r="F46" s="17" t="n"/>
+      <c r="G46" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>산업용라벨프린터</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="E47" s="18" t="n"/>
-      <c r="F47" s="18" t="n"/>
-      <c r="G47" s="18" t="n"/>
-      <c r="H47" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J47" s="20">
-        <f>VLOOKUP(H47,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K47" s="19">
-        <f>IF(J47=0,I47,MAX(I47,MIN($B$10,ROUNDUP(I47*(1+J47),-1))))</f>
-        <v/>
-      </c>
-      <c r="L47" s="21" t="n"/>
-      <c r="M47" s="22">
-        <f>IF(L47&lt;&gt;"",MIN($B$10,L47),K47)</f>
-        <v/>
-      </c>
-      <c r="N47" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="O47" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P47" s="18" t="inlineStr">
-        <is>
-          <t>4,970원</t>
-        </is>
-      </c>
+          <t>제브라</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>산업용바코드프린터</t>
-        </is>
-      </c>
-      <c r="B48" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C48" s="23" t="n">
+          <t>제브라라벨프린터</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D48" s="23" t="n"/>
-      <c r="E48" s="23" t="n"/>
-      <c r="F48" s="23" t="n"/>
-      <c r="G48" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H48" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I48" s="25" t="n">
-        <v>800</v>
-      </c>
-      <c r="J48" s="26">
-        <f>VLOOKUP(H48,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K48" s="25">
-        <f>IF(J48=0,I48,MAX(I48,MIN($B$10,ROUNDUP(I48*(1+J48),-1))))</f>
-        <v/>
-      </c>
-      <c r="L48" s="21" t="n"/>
-      <c r="M48" s="27">
-        <f>IF(L48&lt;&gt;"",MIN($B$10,L48),K48)</f>
-        <v/>
-      </c>
-      <c r="N48" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O48" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="D48" s="17" t="n">
+        <v>700</v>
+      </c>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" s="9" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>산업용프린터</t>
-        </is>
-      </c>
-      <c r="B49" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="n">
+          <t>제브라바코드프린터</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" s="17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E49" s="17" t="n"/>
+      <c r="F49" s="17" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D49" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H49" s="23" t="inlineStr">
-        <is>
-          <t>붙어있음(위)</t>
-        </is>
-      </c>
-      <c r="I49" s="25" t="n">
-        <v>6500</v>
-      </c>
-      <c r="J49" s="26">
-        <f>VLOOKUP(H49,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K49" s="25">
-        <f>IF(J49=0,I49,MAX(I49,MIN($B$10,ROUNDUP(I49*(1+J49),-1))))</f>
-        <v/>
-      </c>
-      <c r="L49" s="21" t="n"/>
-      <c r="M49" s="27">
-        <f>IF(L49&lt;&gt;"",MIN($B$10,L49),K49)</f>
-        <v/>
-      </c>
-      <c r="N49" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="O49" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="P49" s="23" t="inlineStr">
-        <is>
-          <t>6,578원</t>
-        </is>
-      </c>
+      <c r="I49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>소형바코드프린터</t>
-        </is>
-      </c>
-      <c r="B50" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C50" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="D50" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="E50" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="F50" s="23" t="n"/>
-      <c r="G50" s="24" t="inlineStr">
+          <t>제브라프린터</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H50" s="23" t="inlineStr">
-        <is>
-          <t>붙어있음(아래)</t>
-        </is>
-      </c>
-      <c r="I50" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J50" s="26">
-        <f>VLOOKUP(H50,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K50" s="25">
-        <f>IF(J50=0,I50,MAX(I50,MIN($B$10,ROUNDUP(I50*(1+J50),-1))))</f>
-        <v/>
-      </c>
-      <c r="L50" s="21" t="n"/>
-      <c r="M50" s="27">
-        <f>IF(L50&lt;&gt;"",MIN($B$10,L50),K50)</f>
-        <v/>
-      </c>
-      <c r="N50" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P50" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C50" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D50" s="17" t="n">
+        <v>1410</v>
+      </c>
+      <c r="E50" s="17" t="n"/>
+      <c r="F50" s="17" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>스티커라벨기</t>
-        </is>
-      </c>
-      <c r="B51" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C51" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D51" s="23" t="n"/>
-      <c r="E51" s="23" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="24" t="inlineStr">
+          <t>카드프린터기</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H51" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I51" s="25" t="n">
-        <v>2300</v>
-      </c>
-      <c r="J51" s="26">
-        <f>VLOOKUP(H51,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K51" s="25">
-        <f>IF(J51=0,I51,MAX(I51,MIN($B$10,ROUNDUP(I51*(1+J51),-1))))</f>
-        <v/>
-      </c>
-      <c r="L51" s="21" t="n"/>
-      <c r="M51" s="27">
-        <f>IF(L51&lt;&gt;"",MIN($B$10,L51),K51)</f>
-        <v/>
-      </c>
-      <c r="N51" s="23" t="n">
-        <v>21</v>
-      </c>
-      <c r="O51" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P51" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="C51" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D51" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E51" s="17" t="n"/>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>스티커인쇄기</t>
-        </is>
-      </c>
-      <c r="B52" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="D52" s="18" t="n"/>
-      <c r="E52" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="F52" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="18" t="n"/>
-      <c r="H52" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I52" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="J52" s="20">
-        <f>VLOOKUP(H52,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K52" s="19">
-        <f>IF(J52=0,I52,MAX(I52,MIN($B$10,ROUNDUP(I52*(1+J52),-1))))</f>
-        <v/>
-      </c>
-      <c r="L52" s="21" t="n"/>
-      <c r="M52" s="22">
-        <f>IF(L52&lt;&gt;"",MIN($B$10,L52),K52)</f>
-        <v/>
-      </c>
-      <c r="N52" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="O52" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P52" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>스티커출력기</t>
-        </is>
-      </c>
-      <c r="B53" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C53" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D53" s="23" t="n">
+          <t>프린터관리</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="E53" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H53" s="23" t="inlineStr">
-        <is>
-          <t>순위 차이 큼</t>
-        </is>
-      </c>
-      <c r="I53" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="J53" s="26">
-        <f>VLOOKUP(H53,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K53" s="25">
-        <f>IF(J53=0,I53,MAX(I53,MIN($B$10,ROUNDUP(I53*(1+J53),-1))))</f>
-        <v/>
-      </c>
-      <c r="L53" s="21" t="n"/>
-      <c r="M53" s="27">
-        <f>IF(L53&lt;&gt;"",MIN($B$10,L53),K53)</f>
-        <v/>
-      </c>
-      <c r="N53" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="O53" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P53" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>스티커프린터</t>
-        </is>
-      </c>
-      <c r="B54" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C54" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D54" s="23" t="n"/>
-      <c r="E54" s="23" t="n"/>
-      <c r="F54" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H54" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I54" s="25" t="n">
-        <v>1340</v>
-      </c>
-      <c r="J54" s="26">
-        <f>VLOOKUP(H54,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K54" s="25">
-        <f>IF(J54=0,I54,MAX(I54,MIN($B$10,ROUNDUP(I54*(1+J54),-1))))</f>
-        <v/>
-      </c>
-      <c r="L54" s="21" t="n"/>
-      <c r="M54" s="27">
-        <f>IF(L54&lt;&gt;"",MIN($B$10,L54),K54)</f>
-        <v/>
-      </c>
-      <c r="N54" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="O54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>열전사프린터</t>
-        </is>
-      </c>
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C55" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="D55" s="23" t="n"/>
-      <c r="E55" s="23" t="n"/>
-      <c r="F55" s="23" t="n"/>
-      <c r="G55" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H55" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I55" s="25" t="n">
-        <v>5500</v>
-      </c>
-      <c r="J55" s="26">
-        <f>VLOOKUP(H55,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K55" s="25">
-        <f>IF(J55=0,I55,MAX(I55,MIN($B$10,ROUNDUP(I55*(1+J55),-1))))</f>
-        <v/>
-      </c>
-      <c r="L55" s="21" t="n"/>
-      <c r="M55" s="27">
-        <f>IF(L55&lt;&gt;"",MIN($B$10,L55),K55)</f>
-        <v/>
-      </c>
-      <c r="N55" s="23" t="n">
-        <v>13</v>
-      </c>
-      <c r="O55" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>열전사프린터기</t>
-        </is>
-      </c>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C56" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D56" s="23" t="n"/>
-      <c r="E56" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="F56" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="G56" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H56" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I56" s="25" t="n">
-        <v>450</v>
-      </c>
-      <c r="J56" s="26">
-        <f>VLOOKUP(H56,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K56" s="25">
-        <f>IF(J56=0,I56,MAX(I56,MIN($B$10,ROUNDUP(I56*(1+J56),-1))))</f>
-        <v/>
-      </c>
-      <c r="L56" s="21" t="n"/>
-      <c r="M56" s="27">
-        <f>IF(L56&lt;&gt;"",MIN($B$10,L56),K56)</f>
-        <v/>
-      </c>
-      <c r="N56" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P56" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>영수증프린터</t>
-        </is>
-      </c>
-      <c r="B57" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C57" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D57" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="E57" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="F57" s="23" t="n"/>
-      <c r="G57" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H57" s="23" t="inlineStr">
-        <is>
-          <t>붙어있음(위)</t>
-        </is>
-      </c>
-      <c r="I57" s="25" t="n">
-        <v>1070</v>
-      </c>
-      <c r="J57" s="26">
-        <f>VLOOKUP(H57,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K57" s="25">
-        <f>IF(J57=0,I57,MAX(I57,MIN($B$10,ROUNDUP(I57*(1+J57),-1))))</f>
-        <v/>
-      </c>
-      <c r="L57" s="21" t="n"/>
-      <c r="M57" s="27">
-        <f>IF(L57&lt;&gt;"",MIN($B$10,L57),K57)</f>
-        <v/>
-      </c>
-      <c r="N57" s="23" t="n">
-        <v>85</v>
-      </c>
-      <c r="O57" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P57" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
-        <is>
-          <t>제브라</t>
-        </is>
-      </c>
-      <c r="B58" s="18" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C58" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="D58" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="18" t="n"/>
-      <c r="G58" s="18" t="n"/>
-      <c r="H58" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I58" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="J58" s="20">
-        <f>VLOOKUP(H58,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K58" s="19">
-        <f>IF(J58=0,I58,MAX(I58,MIN($B$10,ROUNDUP(I58*(1+J58),-1))))</f>
-        <v/>
-      </c>
-      <c r="L58" s="21" t="n"/>
-      <c r="M58" s="22">
-        <f>IF(L58&lt;&gt;"",MIN($B$10,L58),K58)</f>
-        <v/>
-      </c>
-      <c r="N58" s="18" t="n">
-        <v>115</v>
-      </c>
-      <c r="O58" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="P58" s="18" t="inlineStr">
-        <is>
-          <t>1,464원</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>제브라라벨프린터</t>
-        </is>
-      </c>
-      <c r="B59" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C59" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D59" s="23" t="n"/>
-      <c r="E59" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="F59" s="23" t="n"/>
-      <c r="G59" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H59" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I59" s="25" t="n">
-        <v>700</v>
-      </c>
-      <c r="J59" s="26">
-        <f>VLOOKUP(H59,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K59" s="25">
-        <f>IF(J59=0,I59,MAX(I59,MIN($B$10,ROUNDUP(I59*(1+J59),-1))))</f>
-        <v/>
-      </c>
-      <c r="L59" s="21" t="n"/>
-      <c r="M59" s="27">
-        <f>IF(L59&lt;&gt;"",MIN($B$10,L59),K59)</f>
-        <v/>
-      </c>
-      <c r="N59" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="O59" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t>제브라바코드프린터</t>
-        </is>
-      </c>
-      <c r="B60" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C60" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D60" s="23" t="n"/>
-      <c r="E60" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="F60" s="23" t="n"/>
-      <c r="G60" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H60" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I60" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J60" s="26">
-        <f>VLOOKUP(H60,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K60" s="25">
-        <f>IF(J60=0,I60,MAX(I60,MIN($B$10,ROUNDUP(I60*(1+J60),-1))))</f>
-        <v/>
-      </c>
-      <c r="L60" s="21" t="n"/>
-      <c r="M60" s="27">
-        <f>IF(L60&lt;&gt;"",MIN($B$10,L60),K60)</f>
-        <v/>
-      </c>
-      <c r="N60" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O60" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P60" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>제브라프린터</t>
-        </is>
-      </c>
-      <c r="B61" s="23" t="inlineStr">
-        <is>
-          <t>노출가능</t>
-        </is>
-      </c>
-      <c r="C61" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D61" s="23" t="n"/>
-      <c r="E61" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F61" s="23" t="n"/>
-      <c r="G61" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H61" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I61" s="25" t="n">
-        <v>1410</v>
-      </c>
-      <c r="J61" s="26">
-        <f>VLOOKUP(H61,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K61" s="25">
-        <f>IF(J61=0,I61,MAX(I61,MIN($B$10,ROUNDUP(I61*(1+J61),-1))))</f>
-        <v/>
-      </c>
-      <c r="L61" s="21" t="n"/>
-      <c r="M61" s="27">
-        <f>IF(L61&lt;&gt;"",MIN($B$10,L61),K61)</f>
-        <v/>
-      </c>
-      <c r="N61" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O61" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P61" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>카드프린터기</t>
-        </is>
-      </c>
-      <c r="B62" s="23" t="inlineStr">
-        <is>
-          <t>중지: 키워드 OFF</t>
-        </is>
-      </c>
-      <c r="C62" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="D62" s="23" t="n"/>
-      <c r="E62" s="23" t="n"/>
-      <c r="F62" s="23" t="n"/>
-      <c r="G62" s="24" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="H62" s="23" t="inlineStr">
-        <is>
-          <t>솔바텍 미노출</t>
-        </is>
-      </c>
-      <c r="I62" s="25" t="n">
-        <v>70</v>
-      </c>
-      <c r="J62" s="26">
-        <f>VLOOKUP(H62,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K62" s="25">
-        <f>IF(J62=0,I62,MAX(I62,MIN($B$10,ROUNDUP(I62*(1+J62),-1))))</f>
-        <v/>
-      </c>
-      <c r="L62" s="21" t="n"/>
-      <c r="M62" s="27">
-        <f>IF(L62&lt;&gt;"",MIN($B$10,L62),K62)</f>
-        <v/>
-      </c>
-      <c r="N62" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O62" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P62" s="23" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
-        <is>
-          <t>프린터관리</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>중지: 키워드 OFF</t>
-        </is>
-      </c>
-      <c r="C63" s="18" t="n">
-        <v>7</v>
-      </c>
-      <c r="D63" s="18" t="n"/>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="18" t="n"/>
-      <c r="G63" s="18" t="n"/>
-      <c r="H63" s="18" t="inlineStr">
-        <is>
-          <t>유지</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="n">
+      <c r="D52" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="J63" s="20">
-        <f>VLOOKUP(H63,$A$3:$B$8,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="K63" s="19">
-        <f>IF(J63=0,I63,MAX(I63,MIN($B$10,ROUNDUP(I63*(1+J63),-1))))</f>
-        <v/>
-      </c>
-      <c r="L63" s="21" t="n"/>
-      <c r="M63" s="22">
-        <f>IF(L63&lt;&gt;"",MIN($B$10,L63),K63)</f>
-        <v/>
-      </c>
-      <c r="N63" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="O63" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P63" s="18" t="inlineStr">
-        <is>
-          <t>0원</t>
-        </is>
-      </c>
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="16" t="n"/>
+      <c r="G52" s="7" t="n"/>
+      <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A13:P63"/>
-  <mergeCells count="8">
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C2:F2"/>
+  <autoFilter ref="A2:I52"/>
+  <mergeCells count="5">
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="H14:H63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=$A$3:$A$8</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3767,23 +1947,23 @@
           <t>입찰가 변경 전</t>
         </is>
       </c>
-      <c r="C1" s="28" t="n"/>
-      <c r="D1" s="28" t="n"/>
-      <c r="E1" s="28" t="n"/>
-      <c r="F1" s="28" t="n"/>
-      <c r="G1" s="29" t="n"/>
+      <c r="C1" s="18" t="n"/>
+      <c r="D1" s="18" t="n"/>
+      <c r="E1" s="18" t="n"/>
+      <c r="F1" s="18" t="n"/>
+      <c r="G1" s="19" t="n"/>
       <c r="H1" s="4" t="inlineStr">
         <is>
           <t>입찰가 변경 후</t>
         </is>
       </c>
-      <c r="I1" s="28" t="n"/>
-      <c r="J1" s="28" t="n"/>
-      <c r="K1" s="28" t="n"/>
-      <c r="L1" s="29" t="n"/>
+      <c r="I1" s="18" t="n"/>
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="18" t="n"/>
+      <c r="L1" s="19" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="n"/>
+      <c r="A2" s="20" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>현재 입찰가</t>
@@ -9306,10 +7486,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H305" s="31">
-        <f>'프린터 입찰가'!M21</f>
-        <v/>
-      </c>
+      <c r="H305" s="9" t="n"/>
       <c r="I305" s="9" t="n"/>
       <c r="J305" s="9" t="n"/>
       <c r="K305" s="9" t="n"/>
@@ -9337,10 +7514,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H306" s="31">
-        <f>'프린터 입찰가'!M23</f>
-        <v/>
-      </c>
+      <c r="H306" s="9" t="n"/>
       <c r="I306" s="9" t="n"/>
       <c r="J306" s="9" t="n"/>
       <c r="K306" s="9" t="n"/>
@@ -9368,10 +7542,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H307" s="31">
-        <f>'프린터 입찰가'!M24</f>
-        <v/>
-      </c>
+      <c r="H307" s="9" t="n"/>
       <c r="I307" s="9" t="n"/>
       <c r="J307" s="9" t="n"/>
       <c r="K307" s="9" t="n"/>
@@ -9399,10 +7570,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H308" s="31">
-        <f>'프린터 입찰가'!M26</f>
-        <v/>
-      </c>
+      <c r="H308" s="9" t="n"/>
       <c r="I308" s="9" t="n"/>
       <c r="J308" s="9" t="n"/>
       <c r="K308" s="9" t="n"/>
@@ -9432,10 +7600,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H309" s="31">
-        <f>'프린터 입찰가'!M27</f>
-        <v/>
-      </c>
+      <c r="H309" s="9" t="n"/>
       <c r="I309" s="9" t="n"/>
       <c r="J309" s="9" t="n"/>
       <c r="K309" s="9" t="n"/>
@@ -9463,10 +7628,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H310" s="31">
-        <f>'프린터 입찰가'!M31</f>
-        <v/>
-      </c>
+      <c r="H310" s="9" t="n"/>
       <c r="I310" s="9" t="n"/>
       <c r="J310" s="9" t="n"/>
       <c r="K310" s="9" t="n"/>
@@ -9494,10 +7656,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H311" s="31">
-        <f>'프린터 입찰가'!M36</f>
-        <v/>
-      </c>
+      <c r="H311" s="9" t="n"/>
       <c r="I311" s="9" t="n"/>
       <c r="J311" s="9" t="n"/>
       <c r="K311" s="9" t="n"/>
@@ -9527,10 +7686,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H312" s="31">
-        <f>'프린터 입찰가'!M41</f>
-        <v/>
-      </c>
+      <c r="H312" s="9" t="n"/>
       <c r="I312" s="9" t="n"/>
       <c r="J312" s="9" t="n"/>
       <c r="K312" s="9" t="n"/>
@@ -9582,10 +7738,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H314" s="31">
-        <f>'프린터 입찰가'!M59</f>
-        <v/>
-      </c>
+      <c r="H314" s="9" t="n"/>
       <c r="I314" s="9" t="n"/>
       <c r="J314" s="9" t="n"/>
       <c r="K314" s="9" t="n"/>
@@ -9613,10 +7766,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H315" s="31">
-        <f>'프린터 입찰가'!M60</f>
-        <v/>
-      </c>
+      <c r="H315" s="9" t="n"/>
       <c r="I315" s="9" t="n"/>
       <c r="J315" s="9" t="n"/>
       <c r="K315" s="9" t="n"/>
@@ -9644,10 +7794,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H316" s="31">
-        <f>'프린터 입찰가'!M33</f>
-        <v/>
-      </c>
+      <c r="H316" s="9" t="n"/>
       <c r="I316" s="9" t="n"/>
       <c r="J316" s="9" t="n"/>
       <c r="K316" s="9" t="n"/>
@@ -9675,10 +7822,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H317" s="31">
-        <f>'프린터 입찰가'!M40</f>
-        <v/>
-      </c>
+      <c r="H317" s="9" t="n"/>
       <c r="I317" s="9" t="n"/>
       <c r="J317" s="9" t="n"/>
       <c r="K317" s="9" t="n"/>
@@ -9752,10 +7896,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H320" s="31">
-        <f>'프린터 입찰가'!M20</f>
-        <v/>
-      </c>
+      <c r="H320" s="9" t="n"/>
       <c r="I320" s="9" t="n"/>
       <c r="J320" s="9" t="n"/>
       <c r="K320" s="9" t="n"/>
@@ -9783,10 +7924,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H321" s="31">
-        <f>'프린터 입찰가'!M35</f>
-        <v/>
-      </c>
+      <c r="H321" s="9" t="n"/>
       <c r="I321" s="9" t="n"/>
       <c r="J321" s="9" t="n"/>
       <c r="K321" s="9" t="n"/>
@@ -9814,10 +7952,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H322" s="31">
-        <f>'프린터 입찰가'!M42</f>
-        <v/>
-      </c>
+      <c r="H322" s="9" t="n"/>
       <c r="I322" s="9" t="n"/>
       <c r="J322" s="9" t="n"/>
       <c r="K322" s="9" t="n"/>
@@ -9847,10 +7982,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H323" s="31">
-        <f>'프린터 입찰가'!M46</f>
-        <v/>
-      </c>
+      <c r="H323" s="9" t="n"/>
       <c r="I323" s="9" t="n"/>
       <c r="J323" s="9" t="n"/>
       <c r="K323" s="9" t="n"/>
@@ -9880,10 +8012,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H324" s="31">
-        <f>'프린터 입찰가'!M50</f>
-        <v/>
-      </c>
+      <c r="H324" s="9" t="n"/>
       <c r="I324" s="9" t="n"/>
       <c r="J324" s="9" t="n"/>
       <c r="K324" s="9" t="n"/>
@@ -9935,10 +8064,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H326" s="31">
-        <f>'프린터 입찰가'!M61</f>
-        <v/>
-      </c>
+      <c r="H326" s="9" t="n"/>
       <c r="I326" s="9" t="n"/>
       <c r="J326" s="9" t="n"/>
       <c r="K326" s="9" t="n"/>
@@ -9988,10 +8114,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H328" s="31">
-        <f>'프린터 입찰가'!M45</f>
-        <v/>
-      </c>
+      <c r="H328" s="9" t="n"/>
       <c r="I328" s="9" t="n"/>
       <c r="J328" s="9" t="n"/>
       <c r="K328" s="9" t="n"/>
@@ -10017,10 +8140,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H329" s="31">
-        <f>'프린터 입찰가'!M48</f>
-        <v/>
-      </c>
+      <c r="H329" s="9" t="n"/>
       <c r="I329" s="9" t="n"/>
       <c r="J329" s="9" t="n"/>
       <c r="K329" s="9" t="n"/>
@@ -10050,10 +8170,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H330" s="31">
-        <f>'프린터 입찰가'!M49</f>
-        <v/>
-      </c>
+      <c r="H330" s="9" t="n"/>
       <c r="I330" s="9" t="n"/>
       <c r="J330" s="9" t="n"/>
       <c r="K330" s="9" t="n"/>
@@ -10079,10 +8196,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H331" s="31">
-        <f>'프린터 입찰가'!M51</f>
-        <v/>
-      </c>
+      <c r="H331" s="9" t="n"/>
       <c r="I331" s="9" t="n"/>
       <c r="J331" s="9" t="n"/>
       <c r="K331" s="9" t="n"/>
@@ -10110,10 +8224,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H332" s="31">
-        <f>'프린터 입찰가'!M54</f>
-        <v/>
-      </c>
+      <c r="H332" s="9" t="n"/>
       <c r="I332" s="9" t="n"/>
       <c r="J332" s="9" t="n"/>
       <c r="K332" s="9" t="n"/>
@@ -10169,10 +8280,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H334" s="31">
-        <f>'프린터 입찰가'!M53</f>
-        <v/>
-      </c>
+      <c r="H334" s="9" t="n"/>
       <c r="I334" s="9" t="n"/>
       <c r="J334" s="9" t="n"/>
       <c r="K334" s="9" t="n"/>
@@ -10200,10 +8308,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H335" s="31">
-        <f>'프린터 입찰가'!M30</f>
-        <v/>
-      </c>
+      <c r="H335" s="9" t="n"/>
       <c r="I335" s="9" t="n"/>
       <c r="J335" s="9" t="n"/>
       <c r="K335" s="9" t="n"/>
@@ -10231,10 +8336,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H336" s="31">
-        <f>'프린터 입찰가'!M29</f>
-        <v/>
-      </c>
+      <c r="H336" s="9" t="n"/>
       <c r="I336" s="9" t="n"/>
       <c r="J336" s="9" t="n"/>
       <c r="K336" s="9" t="n"/>
@@ -10262,10 +8364,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H337" s="31">
-        <f>'프린터 입찰가'!M28</f>
-        <v/>
-      </c>
+      <c r="H337" s="9" t="n"/>
       <c r="I337" s="9" t="n"/>
       <c r="J337" s="9" t="n"/>
       <c r="K337" s="9" t="n"/>
@@ -10295,10 +8394,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H338" s="31">
-        <f>'프린터 입찰가'!M57</f>
-        <v/>
-      </c>
+      <c r="H338" s="9" t="n"/>
       <c r="I338" s="9" t="n"/>
       <c r="J338" s="9" t="n"/>
       <c r="K338" s="9" t="n"/>
@@ -10330,10 +8426,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H339" s="31">
-        <f>'프린터 입찰가'!M16</f>
-        <v/>
-      </c>
+      <c r="H339" s="9" t="n"/>
       <c r="I339" s="9" t="n"/>
       <c r="J339" s="9" t="n"/>
       <c r="K339" s="9" t="n"/>
@@ -10363,10 +8456,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H340" s="31">
-        <f>'프린터 입찰가'!M56</f>
-        <v/>
-      </c>
+      <c r="H340" s="9" t="n"/>
       <c r="I340" s="9" t="n"/>
       <c r="J340" s="9" t="n"/>
       <c r="K340" s="9" t="n"/>
@@ -10392,10 +8482,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H341" s="31">
-        <f>'프린터 입찰가'!M55</f>
-        <v/>
-      </c>
+      <c r="H341" s="9" t="n"/>
       <c r="I341" s="9" t="n"/>
       <c r="J341" s="9" t="n"/>
       <c r="K341" s="9" t="n"/>
@@ -10447,10 +8534,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H343" s="31">
-        <f>'프린터 입찰가'!M19</f>
-        <v/>
-      </c>
+      <c r="H343" s="9" t="n"/>
       <c r="I343" s="9" t="n"/>
       <c r="J343" s="9" t="n"/>
       <c r="K343" s="9" t="n"/>
@@ -10482,10 +8566,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H344" s="31">
-        <f>'프린터 입찰가'!M37</f>
-        <v/>
-      </c>
+      <c r="H344" s="9" t="n"/>
       <c r="I344" s="9" t="n"/>
       <c r="J344" s="9" t="n"/>
       <c r="K344" s="9" t="n"/>
@@ -10515,10 +8596,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H345" s="31">
-        <f>'프린터 입찰가'!M25</f>
-        <v/>
-      </c>
+      <c r="H345" s="9" t="n"/>
       <c r="I345" s="9" t="n"/>
       <c r="J345" s="9" t="n"/>
       <c r="K345" s="9" t="n"/>
@@ -10548,10 +8626,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H346" s="31">
-        <f>'프린터 입찰가'!M39</f>
-        <v/>
-      </c>
+      <c r="H346" s="9" t="n"/>
       <c r="I346" s="9" t="n"/>
       <c r="J346" s="9" t="n"/>
       <c r="K346" s="9" t="n"/>
@@ -10579,10 +8654,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H347" s="31">
-        <f>'프린터 입찰가'!M18</f>
-        <v/>
-      </c>
+      <c r="H347" s="9" t="n"/>
       <c r="I347" s="9" t="n"/>
       <c r="J347" s="9" t="n"/>
       <c r="K347" s="9" t="n"/>
@@ -10610,10 +8682,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H348" s="31">
-        <f>'프린터 입찰가'!M38</f>
-        <v/>
-      </c>
+      <c r="H348" s="9" t="n"/>
       <c r="I348" s="9" t="n"/>
       <c r="J348" s="9" t="n"/>
       <c r="K348" s="9" t="n"/>
@@ -10643,10 +8712,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H349" s="31">
-        <f>'프린터 입찰가'!M32</f>
-        <v/>
-      </c>
+      <c r="H349" s="9" t="n"/>
       <c r="I349" s="9" t="n"/>
       <c r="J349" s="9" t="n"/>
       <c r="K349" s="9" t="n"/>
@@ -10674,10 +8740,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H350" s="31">
-        <f>'프린터 입찰가'!M22</f>
-        <v/>
-      </c>
+      <c r="H350" s="9" t="n"/>
       <c r="I350" s="9" t="n"/>
       <c r="J350" s="9" t="n"/>
       <c r="K350" s="9" t="n"/>
@@ -12125,10 +10188,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H430" s="31">
-        <f>'프린터 입찰가'!M34</f>
-        <v/>
-      </c>
+      <c r="H430" s="9" t="n"/>
       <c r="I430" s="9" t="n"/>
       <c r="J430" s="9" t="n"/>
       <c r="K430" s="9" t="n"/>
@@ -12154,10 +10214,7 @@
           <t>수정필요</t>
         </is>
       </c>
-      <c r="H431" s="31">
-        <f>'프린터 입찰가'!M62</f>
-        <v/>
-      </c>
+      <c r="H431" s="9" t="n"/>
       <c r="I431" s="9" t="n"/>
       <c r="J431" s="9" t="n"/>
       <c r="K431" s="9" t="n"/>

</xml_diff>

<commit_message>
Fill Cosmos Mall and SB Rental bids in printer bid sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KT1VW3oarL8CCbJcMVGP8
</commit_message>
<xml_diff>
--- a/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
+++ b/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
@@ -49,7 +49,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE5E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -180,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -217,10 +222,25 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -591,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -603,6 +623,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -635,6 +656,11 @@
       </c>
       <c r="H1" s="5" t="n"/>
       <c r="I1" s="5" t="n"/>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t>범례</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="D2" s="14" t="inlineStr">
@@ -667,107 +693,82 @@
           <t>sb렌탈</t>
         </is>
       </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>회색 칸 = 키워드 OFF(중지)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="K3" s="16" t="inlineStr">
+        <is>
+          <t>굵은 글씨 = 3개 사이트 중 최고 입찰가</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>빨간 글씨 = 입찰가 수정 대상</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>감열식프린터</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n"/>
-      <c r="C3" s="7" t="n">
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D5" s="19" t="n">
         <v>800</v>
       </c>
-      <c r="E3" s="16" t="n"/>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="7" t="n">
+      <c r="E5" s="20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="H5" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="I3" s="7" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>감열프린터</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n"/>
-      <c r="C4" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" s="16" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>감열프린터기</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" s="17" t="n">
-        <v>650</v>
-      </c>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>3</v>
-      </c>
+      <c r="I5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>도시바프린터</t>
+          <t>감열프린터</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E6" s="19" t="n">
         <v>1500</v>
       </c>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
+      <c r="F6" s="19" t="n">
+        <v>1330</v>
+      </c>
       <c r="G6" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
+      <c r="I6" s="7" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>라밸프린터</t>
+          <t>감열프린터기</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -778,44 +779,50 @@
       <c r="C7" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
+      <c r="D7" s="21" t="n">
+        <v>650</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>7</v>
+      </c>
       <c r="I7" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>도시바프린터</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="7" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>라벨기</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="17" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>라벨기계</t>
+          <t>라밸프린터</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -826,19 +833,23 @@
       <c r="C9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>890</v>
-      </c>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n"/>
+      <c r="D9" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F9" s="21" t="n"/>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
+      <c r="I9" s="9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>라벨용지프린터</t>
+          <t>라벨기</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -847,23 +858,23 @@
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="22" t="n">
+        <v>5000</v>
+      </c>
       <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n">
-        <v>3</v>
-      </c>
+      <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기</t>
+          <t>라벨기계</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -874,21 +885,19 @@
       <c r="C11" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D11" s="17" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="17" t="n"/>
+      <c r="D11" s="21" t="n">
+        <v>890</v>
+      </c>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="I11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기계</t>
+          <t>라벨용지프린터</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -897,23 +906,23 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>600</v>
-      </c>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
       <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="H12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>라벨지프린터</t>
+          <t>라벨인쇄기</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -924,21 +933,23 @@
       <c r="C13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D13" s="17" t="n">
-        <v>800</v>
-      </c>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="17" t="n"/>
+      <c r="D13" s="21" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F13" s="21" t="n"/>
       <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>라벨출력기</t>
+          <t>라벨인쇄기계</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -949,23 +960,21 @@
       <c r="C14" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D14" s="17" t="n">
-        <v>1110</v>
-      </c>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H14" s="9" t="n">
+      <c r="D14" s="21" t="n">
+        <v>600</v>
+      </c>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="21" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터업체</t>
+          <t>라벨지프린터</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -976,21 +985,23 @@
       <c r="C15" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D15" s="17" t="n">
-        <v>530</v>
-      </c>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
+      <c r="D15" s="21" t="n">
+        <v>800</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>1790</v>
+      </c>
+      <c r="F15" s="21" t="n"/>
       <c r="G15" s="9" t="n"/>
       <c r="H15" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터추천</t>
+          <t>라벨출력기</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -1001,23 +1012,23 @@
       <c r="C16" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="17" t="n">
-        <v>1580</v>
-      </c>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
+      <c r="D16" s="21" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="21" t="n"/>
       <c r="G16" s="9" t="n">
         <v>7</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>롤라벨인쇄기</t>
+          <t>라벨프린터업체</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -1028,21 +1039,21 @@
       <c r="C17" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D17" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n"/>
+      <c r="D17" s="21" t="n">
+        <v>530</v>
+      </c>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="21" t="n"/>
       <c r="G17" s="9" t="n"/>
       <c r="H17" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>롤라벨출력기</t>
+          <t>라벨프린터추천</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -1051,23 +1062,25 @@
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D18" s="17" t="n">
-        <v>100</v>
-      </c>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="9" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>1580</v>
+      </c>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="9" t="n">
+        <v>7</v>
+      </c>
       <c r="H18" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>롤라벨프린터</t>
+          <t>롤라벨인쇄기</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -1078,21 +1091,23 @@
       <c r="C19" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D19" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H19" s="9" t="n"/>
+      <c r="D19" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="I19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨인쇄기</t>
+          <t>롤라벨출력기</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -1101,13 +1116,15 @@
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D20" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>500</v>
+      </c>
+      <c r="F20" s="21" t="n"/>
       <c r="G20" s="9" t="n"/>
       <c r="H20" s="9" t="n">
         <v>3</v>
@@ -1117,7 +1134,7 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨프린터</t>
+          <t>롤라벨프린터</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1128,23 +1145,23 @@
       <c r="C21" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D21" s="17" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="17" t="n"/>
+      <c r="D21" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F21" s="21" t="n"/>
       <c r="G21" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="H21" s="9" t="n">
-        <v>4</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="H21" s="9" t="n"/>
       <c r="I21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨프린터업체</t>
+          <t>바코드라벨인쇄기</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -1153,13 +1170,13 @@
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D22" s="17" t="n">
-        <v>300</v>
-      </c>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="21" t="n"/>
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="9" t="n">
         <v>3</v>
@@ -1169,7 +1186,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>바코드만들기</t>
+          <t>바코드라벨프린터</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -1178,21 +1195,29 @@
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D23" s="17" t="n">
-        <v>500</v>
-      </c>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>4460</v>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="I23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>바코드발행기</t>
+          <t>바코드라벨프린터업체</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -1201,13 +1226,13 @@
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D24" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="E24" s="17" t="n"/>
-      <c r="F24" s="17" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="D24" s="21" t="n">
+        <v>300</v>
+      </c>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n">
         <v>3</v>
@@ -1217,7 +1242,7 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>바코드인쇄기</t>
+          <t>바코드만들기</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -1226,23 +1251,23 @@
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D25" s="17" t="n">
-        <v>3300</v>
-      </c>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>910</v>
+      </c>
+      <c r="F25" s="21" t="n"/>
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="9" t="n"/>
-      <c r="I25" s="9" t="n">
-        <v>7</v>
-      </c>
+      <c r="I25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>바코드출력기</t>
+          <t>바코드발행기</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -1251,27 +1276,25 @@
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D26" s="17" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E26" s="17" t="n"/>
-      <c r="F26" s="17" t="n"/>
-      <c r="G26" s="9" t="n">
-        <v>8</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="9" t="n"/>
       <c r="H26" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="9" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터기</t>
+          <t>바코드인쇄기</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -1280,23 +1303,27 @@
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D27" s="17" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E27" s="21" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F27" s="22" t="n">
+        <v>5000</v>
+      </c>
       <c r="G27" s="9" t="n"/>
-      <c r="H27" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" s="9" t="n"/>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" s="9" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터라벨</t>
+          <t>바코드출력기</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -1305,25 +1332,31 @@
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D28" s="17" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E28" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F28" s="22" t="n">
+        <v>4000</v>
+      </c>
       <c r="G28" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" s="9" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터전문업체</t>
+          <t>바코드프린터기</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -1332,23 +1365,25 @@
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" s="17" t="n">
-        <v>700</v>
-      </c>
-      <c r="E29" s="17" t="n"/>
-      <c r="F29" s="17" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="D29" s="21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F29" s="21" t="n"/>
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터추천</t>
+          <t>바코드프린터라벨</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -1359,23 +1394,23 @@
       <c r="C30" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D30" s="17" t="n">
-        <v>1700</v>
-      </c>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="9" t="n"/>
+      <c r="D30" s="21" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E30" s="21" t="n"/>
+      <c r="F30" s="21" t="n"/>
+      <c r="G30" s="9" t="n">
+        <v>7</v>
+      </c>
       <c r="H30" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I30" s="9" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터판매</t>
+          <t>바코드프린터전문업체</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -1386,11 +1421,13 @@
       <c r="C31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D31" s="17" t="n">
-        <v>280</v>
-      </c>
-      <c r="E31" s="17" t="n"/>
-      <c r="F31" s="17" t="n"/>
+      <c r="D31" s="21" t="n">
+        <v>700</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F31" s="21" t="n"/>
       <c r="G31" s="9" t="n"/>
       <c r="H31" s="9" t="n">
         <v>2</v>
@@ -1398,122 +1435,132 @@
       <c r="I31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터추천</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F32" s="21" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>바코드프린터판매</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>280</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F33" s="21" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" s="9" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>바코드프린터프로그램</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n">
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D32" s="16" t="n">
+      <c r="D34" s="19" t="n">
         <v>2750</v>
       </c>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="7" t="n">
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="7" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>빅솔론</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n">
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="D33" s="16" t="n">
+      <c r="D35" s="20" t="n">
         <v>800</v>
       </c>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
-      <c r="G33" s="7" t="n">
+      <c r="E35" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="H35" s="7" t="n"/>
+      <c r="I35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>빅솔론총판</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n">
+      <c r="C36" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D36" s="21" t="n">
         <v>70</v>
       </c>
-      <c r="E34" s="17" t="n"/>
-      <c r="F34" s="17" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>빅솔론프린터</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D35" s="17" t="n">
-        <v>940</v>
-      </c>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H35" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I35" s="9" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>산업용라벨프린터</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
+      <c r="E36" s="21" t="n"/>
+      <c r="F36" s="21" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>산업용바코드프린터</t>
+          <t>빅솔론프린터</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
@@ -1524,46 +1571,48 @@
       <c r="C37" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="17" t="n">
-        <v>800</v>
-      </c>
-      <c r="E37" s="17" t="n"/>
-      <c r="F37" s="17" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="9" t="n"/>
+      <c r="D37" s="21" t="n">
+        <v>940</v>
+      </c>
+      <c r="E37" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F37" s="21" t="n"/>
+      <c r="G37" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="I37" s="9" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>산업용프린터</t>
-        </is>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D38" s="17" t="n">
-        <v>6500</v>
-      </c>
-      <c r="E38" s="17" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I38" s="9" t="n"/>
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>산업용라벨프린터</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n"/>
+      <c r="C38" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D38" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H38" s="7" t="n"/>
+      <c r="I38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>소형바코드프린터</t>
+          <t>산업용바코드프린터</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -1572,25 +1621,23 @@
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D39" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E39" s="17" t="n"/>
-      <c r="F39" s="17" t="n"/>
-      <c r="G39" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H39" s="9" t="n">
-        <v>5</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D39" s="21" t="n">
+        <v>800</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F39" s="21" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
       <c r="I39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>스티커라벨기</t>
+          <t>산업용프린터</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
@@ -1599,44 +1646,56 @@
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D40" s="17" t="n">
-        <v>2300</v>
-      </c>
-      <c r="E40" s="17" t="n"/>
-      <c r="F40" s="17" t="n"/>
-      <c r="G40" s="9" t="n"/>
-      <c r="H40" s="9" t="n"/>
+        <v>7</v>
+      </c>
+      <c r="D40" s="21" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E40" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="I40" s="9" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>스티커인쇄기</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D41" s="16" t="n">
-        <v>800</v>
-      </c>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>소형바코드프린터</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D41" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E41" s="22" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F41" s="21" t="n"/>
+      <c r="G41" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="I41" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="I41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>스티커출력기</t>
+          <t>스티커라벨기</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -1645,50 +1704,48 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D42" s="17" t="n">
-        <v>400</v>
-      </c>
-      <c r="E42" s="17" t="n"/>
-      <c r="F42" s="17" t="n"/>
-      <c r="G42" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H42" s="9" t="n">
-        <v>1</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D42" s="22" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E42" s="21" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F42" s="21" t="n"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9" t="n"/>
       <c r="I42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>스티커프린터</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D43" s="17" t="n">
-        <v>1340</v>
-      </c>
-      <c r="E43" s="17" t="n"/>
-      <c r="F43" s="17" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="9" t="n"/>
-      <c r="I43" s="9" t="n">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>스티커인쇄기</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D43" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F43" s="19" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I43" s="7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>열전사프린터</t>
+          <t>스티커출력기</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -1697,21 +1754,27 @@
         </is>
       </c>
       <c r="C44" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E44" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F44" s="21" t="n"/>
+      <c r="G44" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="D44" s="17" t="n">
-        <v>5500</v>
-      </c>
-      <c r="E44" s="17" t="n"/>
-      <c r="F44" s="17" t="n"/>
-      <c r="G44" s="9" t="n"/>
-      <c r="H44" s="9" t="n"/>
+      <c r="H44" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="I44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>열전사프린터기</t>
+          <t>스티커프린터</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -1720,25 +1783,25 @@
         </is>
       </c>
       <c r="C45" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D45" s="17" t="n">
-        <v>450</v>
-      </c>
-      <c r="E45" s="17" t="n"/>
-      <c r="F45" s="17" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D45" s="21" t="n">
+        <v>1340</v>
+      </c>
+      <c r="E45" s="22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F45" s="21" t="n"/>
       <c r="G45" s="9" t="n"/>
-      <c r="H45" s="9" t="n">
-        <v>8</v>
-      </c>
+      <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>영수증프린터</t>
+          <t>열전사프린터</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -1747,46 +1810,56 @@
         </is>
       </c>
       <c r="C46" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D46" s="21" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E46" s="22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F46" s="21" t="n">
+        <v>4550</v>
+      </c>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
+      <c r="I46" s="9" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>열전사프린터기</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" s="21" t="n">
+        <v>450</v>
+      </c>
+      <c r="E47" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D46" s="17" t="n">
-        <v>1070</v>
-      </c>
-      <c r="E46" s="17" t="n"/>
-      <c r="F46" s="17" t="n"/>
-      <c r="G46" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I46" s="9" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>제브라</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="n"/>
-      <c r="C47" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D47" s="16" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E47" s="16" t="n"/>
-      <c r="F47" s="16" t="n"/>
-      <c r="G47" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H47" s="7" t="n"/>
-      <c r="I47" s="7" t="n"/>
+      <c r="I47" s="9" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>제브라라벨프린터</t>
+          <t>영수증프린터</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -1795,48 +1868,48 @@
         </is>
       </c>
       <c r="C48" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D48" s="17" t="n">
-        <v>700</v>
-      </c>
-      <c r="E48" s="17" t="n"/>
-      <c r="F48" s="17" t="n"/>
-      <c r="G48" s="9" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D48" s="21" t="n">
+        <v>1070</v>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F48" s="21" t="n"/>
+      <c r="G48" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="H48" s="9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I48" s="9" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>제브라바코드프린터</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="n">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>제브라</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D49" s="17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E49" s="17" t="n"/>
-      <c r="F49" s="17" t="n"/>
-      <c r="G49" s="9" t="n"/>
-      <c r="H49" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I49" s="9" t="n"/>
+      <c r="D49" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E49" s="19" t="n"/>
+      <c r="F49" s="19" t="n"/>
+      <c r="G49" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H49" s="7" t="n"/>
+      <c r="I49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>제브라프린터</t>
+          <t>제브라라벨프린터</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -1847,21 +1920,23 @@
       <c r="C50" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D50" s="17" t="n">
-        <v>1410</v>
-      </c>
-      <c r="E50" s="17" t="n"/>
-      <c r="F50" s="17" t="n"/>
+      <c r="D50" s="21" t="n">
+        <v>700</v>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F50" s="21" t="n"/>
       <c r="G50" s="9" t="n"/>
       <c r="H50" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>카드프린터기</t>
+          <t>제브라바코드프린터</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -1872,33 +1947,434 @@
       <c r="C51" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D51" s="17" t="n">
+      <c r="D51" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F51" s="21" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I51" s="9" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>제브라프린터</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="21" t="n">
+        <v>1410</v>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F52" s="21" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I52" s="9" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>카드프린터기</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D53" s="23" t="n">
         <v>70</v>
       </c>
-      <c r="E51" s="17" t="n"/>
-      <c r="F51" s="17" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="E53" s="21" t="n"/>
+      <c r="F53" s="21" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="9" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>프린터관리</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="7" t="n">
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D52" s="16" t="n">
+      <c r="D54" s="23" t="n">
         <v>200</v>
       </c>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="16" t="n"/>
-      <c r="G52" s="7" t="n"/>
-      <c r="H52" s="7" t="n"/>
-      <c r="I52" s="7" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="7" t="n"/>
+      <c r="H54" s="7" t="n"/>
+      <c r="I54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>솔바텍에 없는 키워드 (20개)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>B-FV4T</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="19" t="n"/>
+      <c r="E56" s="19" t="n"/>
+      <c r="F56" s="19" t="n">
+        <v>850</v>
+      </c>
+      <c r="G56" s="7" t="n"/>
+      <c r="H56" s="7" t="n"/>
+      <c r="I56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>B-FV4T-GS</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="19" t="n"/>
+      <c r="E57" s="19" t="n"/>
+      <c r="F57" s="19" t="n">
+        <v>90</v>
+      </c>
+      <c r="G57" s="7" t="n"/>
+      <c r="H57" s="7" t="n"/>
+      <c r="I57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>B-FV4T-TS</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n"/>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="19" t="n"/>
+      <c r="E58" s="19" t="n"/>
+      <c r="F58" s="19" t="n">
+        <v>70</v>
+      </c>
+      <c r="G58" s="7" t="n"/>
+      <c r="H58" s="7" t="n"/>
+      <c r="I58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>G530+</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="19" t="n"/>
+      <c r="E59" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F59" s="19" t="n"/>
+      <c r="G59" s="7" t="n"/>
+      <c r="H59" s="7" t="n"/>
+      <c r="I59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>SLPTX400</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="19" t="n"/>
+      <c r="E60" s="19" t="n"/>
+      <c r="F60" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G60" s="7" t="n"/>
+      <c r="H60" s="7" t="n"/>
+      <c r="I60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>SLPTX403</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n"/>
+      <c r="C61" s="7" t="n"/>
+      <c r="D61" s="19" t="n"/>
+      <c r="E61" s="19" t="n"/>
+      <c r="F61" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G61" s="7" t="n"/>
+      <c r="H61" s="7" t="n"/>
+      <c r="I61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>TSC프린터</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="19" t="n"/>
+      <c r="E62" s="23" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F62" s="19" t="n"/>
+      <c r="G62" s="7" t="n"/>
+      <c r="H62" s="7" t="n"/>
+      <c r="I62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>고덱스</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="n"/>
+      <c r="C63" s="7" t="n"/>
+      <c r="D63" s="19" t="n"/>
+      <c r="E63" s="19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F63" s="19" t="n"/>
+      <c r="G63" s="7" t="n"/>
+      <c r="H63" s="7" t="n"/>
+      <c r="I63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>라벨발행기</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="19" t="n"/>
+      <c r="E64" s="19" t="n">
+        <v>2620</v>
+      </c>
+      <c r="F64" s="19" t="n"/>
+      <c r="G64" s="7" t="n"/>
+      <c r="H64" s="7" t="n"/>
+      <c r="I64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>라벨프린터기</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="n"/>
+      <c r="C65" s="7" t="n"/>
+      <c r="D65" s="19" t="n"/>
+      <c r="E65" s="19" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F65" s="19" t="n"/>
+      <c r="G65" s="7" t="n"/>
+      <c r="H65" s="7" t="n"/>
+      <c r="I65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>라벨프린터용지</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="19" t="n"/>
+      <c r="E66" s="19" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F66" s="19" t="n"/>
+      <c r="G66" s="7" t="n"/>
+      <c r="H66" s="7" t="n"/>
+      <c r="I66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>롤프린터</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="19" t="n"/>
+      <c r="E67" s="19" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F67" s="19" t="n"/>
+      <c r="G67" s="7" t="n"/>
+      <c r="H67" s="7" t="n"/>
+      <c r="I67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>바코드구입</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="n"/>
+      <c r="C68" s="7" t="n"/>
+      <c r="D68" s="19" t="n"/>
+      <c r="E68" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F68" s="19" t="n"/>
+      <c r="G68" s="7" t="n"/>
+      <c r="H68" s="7" t="n"/>
+      <c r="I68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>바코드등록</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="n"/>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="19" t="n"/>
+      <c r="E69" s="19" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F69" s="19" t="n"/>
+      <c r="G69" s="7" t="n"/>
+      <c r="H69" s="7" t="n"/>
+      <c r="I69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>바코드라벨프린터기</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="n"/>
+      <c r="C70" s="7" t="n"/>
+      <c r="D70" s="19" t="n"/>
+      <c r="E70" s="19" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F70" s="19" t="n"/>
+      <c r="G70" s="7" t="n"/>
+      <c r="H70" s="7" t="n"/>
+      <c r="I70" s="7" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>바코드생성</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="n"/>
+      <c r="C71" s="7" t="n"/>
+      <c r="D71" s="19" t="n"/>
+      <c r="E71" s="19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F71" s="19" t="n"/>
+      <c r="G71" s="7" t="n"/>
+      <c r="H71" s="7" t="n"/>
+      <c r="I71" s="7" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>바코드프린트</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="n"/>
+      <c r="C72" s="7" t="n"/>
+      <c r="D72" s="19" t="n"/>
+      <c r="E72" s="19" t="n">
+        <v>1520</v>
+      </c>
+      <c r="F72" s="19" t="n"/>
+      <c r="G72" s="7" t="n"/>
+      <c r="H72" s="7" t="n"/>
+      <c r="I72" s="7" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>산업용바코드</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="n"/>
+      <c r="C73" s="7" t="n"/>
+      <c r="D73" s="19" t="n"/>
+      <c r="E73" s="19" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F73" s="19" t="n"/>
+      <c r="G73" s="7" t="n"/>
+      <c r="H73" s="7" t="n"/>
+      <c r="I73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>소형라벨프린터</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="n"/>
+      <c r="C74" s="7" t="n"/>
+      <c r="D74" s="19" t="n"/>
+      <c r="E74" s="19" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F74" s="19" t="n"/>
+      <c r="G74" s="7" t="n"/>
+      <c r="H74" s="7" t="n"/>
+      <c r="I74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>지브라프린터</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="n"/>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="19" t="n"/>
+      <c r="E75" s="19" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F75" s="19" t="n"/>
+      <c r="G75" s="7" t="n"/>
+      <c r="H75" s="7" t="n"/>
+      <c r="I75" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:I52"/>
@@ -1947,23 +2423,23 @@
           <t>입찰가 변경 전</t>
         </is>
       </c>
-      <c r="C1" s="18" t="n"/>
-      <c r="D1" s="18" t="n"/>
-      <c r="E1" s="18" t="n"/>
-      <c r="F1" s="18" t="n"/>
-      <c r="G1" s="19" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="25" t="n"/>
+      <c r="F1" s="25" t="n"/>
+      <c r="G1" s="26" t="n"/>
       <c r="H1" s="4" t="inlineStr">
         <is>
           <t>입찰가 변경 후</t>
         </is>
       </c>
-      <c r="I1" s="18" t="n"/>
-      <c r="J1" s="18" t="n"/>
-      <c r="K1" s="18" t="n"/>
-      <c r="L1" s="19" t="n"/>
+      <c r="I1" s="25" t="n"/>
+      <c r="J1" s="25" t="n"/>
+      <c r="K1" s="25" t="n"/>
+      <c r="L1" s="26" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="n"/>
+      <c r="A2" s="27" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>현재 입찰가</t>

</xml_diff>

<commit_message>
Fix blank rows at top of printer bid sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KT1VW3oarL8CCbJcMVGP8
</commit_message>
<xml_diff>
--- a/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
+++ b/솔바텍_URL도메인변경완료_순위반영_20261029.xlsx
@@ -224,13 +224,13 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -700,6 +700,29 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>감열식프린터</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="E3" s="19" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" s="7" t="n"/>
       <c r="K3" s="16" t="inlineStr">
         <is>
           <t>굵은 글씨 = 3개 사이트 중 최고 입찰가</t>
@@ -707,68 +730,95 @@
       </c>
     </row>
     <row r="4">
-      <c r="K4" s="18" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>감열프린터</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="19" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F4" s="18" t="n">
+        <v>1330</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
         <is>
           <t>빨간 글씨 = 입찰가 수정 대상</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>감열식프린터</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>감열프린터기</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D5" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="E5" s="20" t="n">
+      <c r="D5" s="21" t="n">
+        <v>650</v>
+      </c>
+      <c r="E5" s="21" t="n">
         <v>1500</v>
       </c>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="7" t="n"/>
+      <c r="F5" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>감열프린터</t>
+          <t>도시바프린터</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="20" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E6" s="19" t="n">
+      <c r="D6" s="18" t="n">
         <v>1500</v>
       </c>
-      <c r="F6" s="19" t="n">
-        <v>1330</v>
-      </c>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
       <c r="G6" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n">
-        <v>5</v>
-      </c>
+      <c r="I6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>감열프린터기</t>
+          <t>라밸프린터</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -780,49 +830,47 @@
         <v>8</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>650</v>
-      </c>
-      <c r="E7" s="21" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F7" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>라벨기</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="21" t="n">
         <v>2000</v>
       </c>
-      <c r="G7" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I7" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>도시바프린터</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>라밸프린터</t>
+          <t>라벨기계</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -834,22 +882,18 @@
         <v>8</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E9" s="22" t="n">
-        <v>1700</v>
-      </c>
+        <v>890</v>
+      </c>
+      <c r="E9" s="21" t="n"/>
       <c r="F9" s="21" t="n"/>
       <c r="G9" s="9" t="n"/>
       <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="I9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>라벨기</t>
+          <t>라벨용지프린터</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -858,23 +902,23 @@
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="E10" s="21" t="n"/>
-      <c r="F10" s="22" t="n">
-        <v>5000</v>
-      </c>
+      <c r="F10" s="21" t="n"/>
       <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
+      <c r="H10" s="9" t="n">
+        <v>3</v>
+      </c>
       <c r="I10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>라벨기계</t>
+          <t>라벨인쇄기</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -886,18 +930,22 @@
         <v>8</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>890</v>
-      </c>
-      <c r="E11" s="21" t="n"/>
+        <v>3500</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>5000</v>
+      </c>
       <c r="F11" s="21" t="n"/>
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
+      <c r="I11" s="9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>라벨용지프린터</t>
+          <t>라벨인쇄기계</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -906,23 +954,23 @@
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="E12" s="21" t="n"/>
       <c r="F12" s="21" t="n"/>
       <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기</t>
+          <t>라벨지프린터</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -934,22 +982,22 @@
         <v>8</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>3500</v>
+        <v>800</v>
       </c>
       <c r="E13" s="22" t="n">
-        <v>5000</v>
+        <v>1790</v>
       </c>
       <c r="F13" s="21" t="n"/>
       <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n">
-        <v>2</v>
-      </c>
+      <c r="H13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>라벨인쇄기계</t>
+          <t>라벨출력기</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
@@ -961,20 +1009,22 @@
         <v>8</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>600</v>
+        <v>1110</v>
       </c>
       <c r="E14" s="21" t="n"/>
       <c r="F14" s="21" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n">
+      <c r="G14" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="9" t="n">
         <v>2</v>
       </c>
+      <c r="I14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>라벨지프린터</t>
+          <t>라벨프린터업체</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -986,22 +1036,20 @@
         <v>8</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>800</v>
-      </c>
-      <c r="E15" s="22" t="n">
-        <v>1790</v>
-      </c>
+        <v>530</v>
+      </c>
+      <c r="E15" s="21" t="n"/>
       <c r="F15" s="21" t="n"/>
       <c r="G15" s="9" t="n"/>
       <c r="H15" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>라벨출력기</t>
+          <t>라벨프린터추천</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -1013,7 +1061,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>1110</v>
+        <v>1580</v>
       </c>
       <c r="E16" s="21" t="n"/>
       <c r="F16" s="21" t="n"/>
@@ -1021,14 +1069,14 @@
         <v>7</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터업체</t>
+          <t>롤라벨인쇄기</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -1040,20 +1088,22 @@
         <v>8</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>530</v>
-      </c>
-      <c r="E17" s="21" t="n"/>
+        <v>70</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>4000</v>
+      </c>
       <c r="F17" s="21" t="n"/>
       <c r="G17" s="9" t="n"/>
       <c r="H17" s="9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>라벨프린터추천</t>
+          <t>롤라벨출력기</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -1062,25 +1112,25 @@
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>1580</v>
-      </c>
-      <c r="E18" s="21" t="n"/>
+        <v>100</v>
+      </c>
+      <c r="E18" s="22" t="n">
+        <v>500</v>
+      </c>
       <c r="F18" s="21" t="n"/>
-      <c r="G18" s="9" t="n">
-        <v>7</v>
-      </c>
+      <c r="G18" s="9" t="n"/>
       <c r="H18" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>롤라벨인쇄기</t>
+          <t>롤라벨프린터</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -1092,22 +1142,22 @@
         <v>8</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>70</v>
+        <v>1000</v>
       </c>
       <c r="E19" s="22" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="F19" s="21" t="n"/>
-      <c r="G19" s="9" t="n"/>
-      <c r="H19" s="9" t="n">
-        <v>1</v>
-      </c>
+      <c r="G19" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H19" s="9" t="n"/>
       <c r="I19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>롤라벨출력기</t>
+          <t>바코드라벨인쇄기</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -1116,14 +1166,12 @@
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>100</v>
-      </c>
-      <c r="E20" s="22" t="n">
-        <v>500</v>
-      </c>
+        <v>400</v>
+      </c>
+      <c r="E20" s="21" t="n"/>
       <c r="F20" s="21" t="n"/>
       <c r="G20" s="9" t="n"/>
       <c r="H20" s="9" t="n">
@@ -1134,7 +1182,7 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>롤라벨프린터</t>
+          <t>바코드라벨프린터</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1146,22 +1194,26 @@
         <v>8</v>
       </c>
       <c r="D21" s="21" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E21" s="22" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F21" s="21" t="n"/>
+        <v>3000</v>
+      </c>
+      <c r="E21" s="21" t="n">
+        <v>4460</v>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>5000</v>
+      </c>
       <c r="G21" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H21" s="9" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>4</v>
+      </c>
       <c r="I21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨인쇄기</t>
+          <t>바코드라벨프린터업체</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
@@ -1170,10 +1222,10 @@
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E22" s="21" t="n"/>
       <c r="F22" s="21" t="n"/>
@@ -1186,7 +1238,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨프린터</t>
+          <t>바코드만들기</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -1195,29 +1247,23 @@
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D23" s="21" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E23" s="21" t="n">
-        <v>4460</v>
-      </c>
-      <c r="F23" s="22" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>4</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="D23" s="23" t="n">
+        <v>500</v>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>910</v>
+      </c>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
       <c r="I23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>바코드라벨프린터업체</t>
+          <t>바코드발행기</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -1226,12 +1272,14 @@
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>300</v>
-      </c>
-      <c r="E24" s="21" t="n"/>
+        <v>400</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>1000</v>
+      </c>
       <c r="F24" s="21" t="n"/>
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n">
@@ -1242,7 +1290,7 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>바코드만들기</t>
+          <t>바코드인쇄기</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -1251,23 +1299,27 @@
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D25" s="23" t="n">
-        <v>500</v>
-      </c>
-      <c r="E25" s="24" t="n">
-        <v>910</v>
-      </c>
-      <c r="F25" s="21" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="D25" s="21" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>5000</v>
+      </c>
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="9" t="n"/>
-      <c r="I25" s="9" t="n"/>
+      <c r="I25" s="9" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>바코드발행기</t>
+          <t>바코드출력기</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -1276,25 +1328,31 @@
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D26" s="21" t="n">
-        <v>400</v>
-      </c>
-      <c r="E26" s="22" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F26" s="21" t="n"/>
-      <c r="G26" s="9" t="n"/>
+        <v>2500</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>8</v>
+      </c>
       <c r="H26" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I26" s="9" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>바코드인쇄기</t>
+          <t>바코드프린터기</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -1303,27 +1361,25 @@
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>3300</v>
-      </c>
-      <c r="E27" s="21" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F27" s="22" t="n">
-        <v>5000</v>
-      </c>
+        <v>4000</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F27" s="21" t="n"/>
       <c r="G27" s="9" t="n"/>
-      <c r="H27" s="9" t="n"/>
-      <c r="I27" s="9" t="n">
-        <v>7</v>
-      </c>
+      <c r="H27" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>바코드출력기</t>
+          <t>바코드프린터라벨</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -1332,31 +1388,25 @@
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E28" s="21" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F28" s="22" t="n">
-        <v>4000</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
       <c r="G28" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I28" s="9" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터기</t>
+          <t>바코드프린터전문업체</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -1365,25 +1415,25 @@
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D29" s="21" t="n">
-        <v>4000</v>
+        <v>700</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>15000</v>
+        <v>2000</v>
       </c>
       <c r="F29" s="21" t="n"/>
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터라벨</t>
+          <t>바코드프린터추천</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -1395,22 +1445,24 @@
         <v>7</v>
       </c>
       <c r="D30" s="21" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E30" s="21" t="n"/>
+        <v>1700</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <v>2000</v>
+      </c>
       <c r="F30" s="21" t="n"/>
-      <c r="G30" s="9" t="n">
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="H30" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I30" s="9" t="n"/>
+      <c r="I30" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>바코드프린터전문업체</t>
+          <t>바코드프린터판매</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
@@ -1422,7 +1474,7 @@
         <v>3</v>
       </c>
       <c r="D31" s="21" t="n">
-        <v>700</v>
+        <v>280</v>
       </c>
       <c r="E31" s="22" t="n">
         <v>2000</v>
@@ -1435,132 +1487,128 @@
       <c r="I31" s="9" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>바코드프린터추천</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>바코드프린터프로그램</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" s="18" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E32" s="18" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>빅솔론</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n"/>
+      <c r="C33" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>800</v>
+      </c>
+      <c r="E33" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="7" t="n"/>
+      <c r="I33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>빅솔론총판</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>수정필요</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D32" s="21" t="n">
-        <v>1700</v>
-      </c>
-      <c r="E32" s="22" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F32" s="21" t="n"/>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I32" s="9" t="n">
+      <c r="C34" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>70</v>
+      </c>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" s="9" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>빅솔론프린터</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>940</v>
+      </c>
+      <c r="E35" s="22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F35" s="21" t="n"/>
+      <c r="G35" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" s="9" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>바코드프린터판매</t>
-        </is>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="21" t="n">
-        <v>280</v>
-      </c>
-      <c r="E33" s="22" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F33" s="21" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I33" s="9" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>바코드프린터프로그램</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D34" s="19" t="n">
-        <v>2750</v>
-      </c>
-      <c r="E34" s="19" t="n"/>
-      <c r="F34" s="19" t="n"/>
-      <c r="G34" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="7" t="n"/>
-      <c r="I34" s="7" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>빅솔론</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n">
+      <c r="I35" s="9" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>산업용라벨프린터</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n"/>
+      <c r="C36" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="D35" s="20" t="n">
-        <v>800</v>
-      </c>
-      <c r="E35" s="23" t="n">
-        <v>300</v>
-      </c>
-      <c r="F35" s="19" t="n"/>
-      <c r="G35" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>빅솔론총판</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" s="21" t="n">
-        <v>70</v>
-      </c>
-      <c r="E36" s="21" t="n"/>
-      <c r="F36" s="21" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
-      <c r="I36" s="9" t="n"/>
+      <c r="D36" s="18" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" s="7" t="n"/>
+      <c r="I36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>빅솔론프린터</t>
+          <t>산업용바코드프린터</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
@@ -1572,47 +1620,49 @@
         <v>10</v>
       </c>
       <c r="D37" s="21" t="n">
-        <v>940</v>
+        <v>800</v>
       </c>
       <c r="E37" s="22" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="F37" s="21" t="n"/>
-      <c r="G37" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" s="9" t="n">
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
+      <c r="I37" s="9" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>산업용프린터</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F38" s="21" t="n"/>
+      <c r="G38" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I37" s="9" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>산업용라벨프린터</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D38" s="19" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>8500</v>
-      </c>
-      <c r="F38" s="19" t="n"/>
-      <c r="G38" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
+      <c r="H38" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>산업용바코드프린터</t>
+          <t>소형바코드프린터</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -1621,23 +1671,27 @@
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D39" s="21" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="E39" s="22" t="n">
-        <v>3500</v>
+        <v>1500</v>
       </c>
       <c r="F39" s="21" t="n"/>
-      <c r="G39" s="9" t="n"/>
-      <c r="H39" s="9" t="n"/>
+      <c r="G39" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="I39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>산업용프린터</t>
+          <t>스티커라벨기</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
@@ -1646,56 +1700,48 @@
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D40" s="21" t="n">
-        <v>6500</v>
-      </c>
-      <c r="E40" s="22" t="n">
-        <v>15000</v>
+        <v>10</v>
+      </c>
+      <c r="D40" s="22" t="n">
+        <v>2300</v>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>2000</v>
       </c>
       <c r="F40" s="21" t="n"/>
-      <c r="G40" s="9" t="n">
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>스티커인쇄기</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D41" s="18" t="n">
+        <v>800</v>
+      </c>
+      <c r="E41" s="19" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="7" t="n"/>
+      <c r="H41" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I41" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H40" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I40" s="9" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>소형바코드프린터</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D41" s="21" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E41" s="22" t="n">
-        <v>1500</v>
-      </c>
-      <c r="F41" s="21" t="n"/>
-      <c r="G41" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="H41" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>스티커라벨기</t>
+          <t>스티커출력기</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -1704,48 +1750,54 @@
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D42" s="22" t="n">
-        <v>2300</v>
-      </c>
-      <c r="E42" s="21" t="n">
-        <v>2000</v>
+        <v>8</v>
+      </c>
+      <c r="D42" s="21" t="n">
+        <v>400</v>
+      </c>
+      <c r="E42" s="22" t="n">
+        <v>4000</v>
       </c>
       <c r="F42" s="21" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
+      <c r="G42" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="I42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>스티커인쇄기</t>
-        </is>
-      </c>
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D43" s="19" t="n">
-        <v>800</v>
-      </c>
-      <c r="E43" s="20" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F43" s="19" t="n"/>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I43" s="7" t="n">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>스티커프린터</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" s="21" t="n">
+        <v>1340</v>
+      </c>
+      <c r="E43" s="22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
+      <c r="I43" s="9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>스티커출력기</t>
+          <t>열전사프린터</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -1754,27 +1806,25 @@
         </is>
       </c>
       <c r="C44" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" s="21" t="n">
-        <v>400</v>
+        <v>5500</v>
       </c>
       <c r="E44" s="22" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F44" s="21" t="n"/>
-      <c r="G44" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H44" s="9" t="n">
-        <v>1</v>
-      </c>
+        <v>6000</v>
+      </c>
+      <c r="F44" s="21" t="n">
+        <v>4550</v>
+      </c>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
       <c r="I44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>스티커프린터</t>
+          <t>열전사프린터기</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -1783,25 +1833,29 @@
         </is>
       </c>
       <c r="C45" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" s="21" t="n">
+        <v>450</v>
+      </c>
+      <c r="E45" s="22" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F45" s="21" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D45" s="21" t="n">
-        <v>1340</v>
-      </c>
-      <c r="E45" s="22" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F45" s="21" t="n"/>
-      <c r="G45" s="9" t="n"/>
-      <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>열전사프린터</t>
+          <t>영수증프린터</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -1810,56 +1864,48 @@
         </is>
       </c>
       <c r="C46" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D46" s="21" t="n">
-        <v>5500</v>
+        <v>1070</v>
       </c>
       <c r="E46" s="22" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F46" s="21" t="n">
-        <v>4550</v>
-      </c>
-      <c r="G46" s="9" t="n"/>
-      <c r="H46" s="9" t="n"/>
+        <v>1300</v>
+      </c>
+      <c r="F46" s="21" t="n"/>
+      <c r="G46" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>5</v>
+      </c>
       <c r="I46" s="9" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>열전사프린터기</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D47" s="21" t="n">
-        <v>450</v>
-      </c>
-      <c r="E47" s="22" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="9" t="n">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>제브라</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n"/>
+      <c r="C47" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I47" s="9" t="n">
-        <v>9</v>
-      </c>
+      <c r="D47" s="18" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E47" s="18" t="n"/>
+      <c r="F47" s="18" t="n"/>
+      <c r="G47" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="7" t="n"/>
+      <c r="I47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>영수증프린터</t>
+          <t>제브라라벨프린터</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -1868,48 +1914,52 @@
         </is>
       </c>
       <c r="C48" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D48" s="21" t="n">
+        <v>700</v>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F48" s="21" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I48" s="9" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>제브라바코드프린터</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>수정필요</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D48" s="21" t="n">
-        <v>1070</v>
-      </c>
-      <c r="E48" s="22" t="n">
-        <v>1300</v>
-      </c>
-      <c r="F48" s="21" t="n"/>
-      <c r="G48" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="H48" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I48" s="9" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>제브라</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D49" s="19" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E49" s="19" t="n"/>
-      <c r="F49" s="19" t="n"/>
-      <c r="G49" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
+      <c r="D49" s="21" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F49" s="21" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>제브라라벨프린터</t>
+          <t>제브라프린터</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -1921,22 +1971,22 @@
         <v>10</v>
       </c>
       <c r="D50" s="21" t="n">
-        <v>700</v>
+        <v>1410</v>
       </c>
       <c r="E50" s="22" t="n">
-        <v>1000</v>
+        <v>6000</v>
       </c>
       <c r="F50" s="21" t="n"/>
       <c r="G50" s="9" t="n"/>
       <c r="H50" s="9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>제브라바코드프린터</t>
+          <t>카드프린터기</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -1947,107 +1997,87 @@
       <c r="C51" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="D51" s="21" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>2000</v>
-      </c>
+      <c r="D51" s="23" t="n">
+        <v>70</v>
+      </c>
+      <c r="E51" s="21" t="n"/>
       <c r="F51" s="21" t="n"/>
       <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n">
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>프린터관리</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="I51" s="9" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
-        <is>
-          <t>제브라프린터</t>
-        </is>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="D52" s="21" t="n">
-        <v>1410</v>
-      </c>
-      <c r="E52" s="22" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F52" s="21" t="n"/>
-      <c r="G52" s="9" t="n"/>
-      <c r="H52" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="I52" s="9" t="n"/>
+      <c r="D52" s="23" t="n">
+        <v>200</v>
+      </c>
+      <c r="E52" s="18" t="n"/>
+      <c r="F52" s="18" t="n"/>
+      <c r="G52" s="7" t="n"/>
+      <c r="H52" s="7" t="n"/>
+      <c r="I52" s="7" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>카드프린터기</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t>수정필요</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="D53" s="23" t="n">
-        <v>70</v>
-      </c>
-      <c r="E53" s="21" t="n"/>
-      <c r="F53" s="21" t="n"/>
-      <c r="G53" s="9" t="n"/>
-      <c r="H53" s="9" t="n"/>
-      <c r="I53" s="9" t="n"/>
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>솔바텍에 없는 키워드 (20개)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>프린터관리</t>
+          <t>B-FV4T</t>
         </is>
       </c>
       <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D54" s="23" t="n">
-        <v>200</v>
-      </c>
-      <c r="E54" s="19" t="n"/>
-      <c r="F54" s="19" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="18" t="n"/>
+      <c r="E54" s="18" t="n"/>
+      <c r="F54" s="18" t="n">
+        <v>850</v>
+      </c>
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
       <c r="I54" s="7" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <t>솔바텍에 없는 키워드 (20개)</t>
-        </is>
-      </c>
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>B-FV4T-GS</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="18" t="n"/>
+      <c r="E55" s="18" t="n"/>
+      <c r="F55" s="18" t="n">
+        <v>90</v>
+      </c>
+      <c r="G55" s="7" t="n"/>
+      <c r="H55" s="7" t="n"/>
+      <c r="I55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>B-FV4T</t>
+          <t>B-FV4T-TS</t>
         </is>
       </c>
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
-      <c r="D56" s="19" t="n"/>
-      <c r="E56" s="19" t="n"/>
-      <c r="F56" s="19" t="n">
-        <v>850</v>
+      <c r="D56" s="18" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="18" t="n">
+        <v>70</v>
       </c>
       <c r="G56" s="7" t="n"/>
       <c r="H56" s="7" t="n"/>
@@ -2056,16 +2086,16 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>B-FV4T-GS</t>
+          <t>G530+</t>
         </is>
       </c>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
-      <c r="D57" s="19" t="n"/>
-      <c r="E57" s="19" t="n"/>
-      <c r="F57" s="19" t="n">
-        <v>90</v>
-      </c>
+      <c r="D57" s="18" t="n"/>
+      <c r="E57" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F57" s="18" t="n"/>
       <c r="G57" s="7" t="n"/>
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="7" t="n"/>
@@ -2073,15 +2103,15 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>B-FV4T-TS</t>
+          <t>SLPTX400</t>
         </is>
       </c>
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
-      <c r="D58" s="19" t="n"/>
-      <c r="E58" s="19" t="n"/>
-      <c r="F58" s="19" t="n">
-        <v>70</v>
+      <c r="D58" s="18" t="n"/>
+      <c r="E58" s="18" t="n"/>
+      <c r="F58" s="18" t="n">
+        <v>1500</v>
       </c>
       <c r="G58" s="7" t="n"/>
       <c r="H58" s="7" t="n"/>
@@ -2090,16 +2120,16 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>G530+</t>
+          <t>SLPTX403</t>
         </is>
       </c>
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="19" t="n"/>
-      <c r="E59" s="19" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F59" s="19" t="n"/>
+      <c r="D59" s="18" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="18" t="n">
+        <v>1500</v>
+      </c>
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
@@ -2107,16 +2137,16 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>SLPTX400</t>
+          <t>TSC프린터</t>
         </is>
       </c>
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
-      <c r="D60" s="19" t="n"/>
-      <c r="E60" s="19" t="n"/>
-      <c r="F60" s="19" t="n">
-        <v>1500</v>
-      </c>
+      <c r="D60" s="18" t="n"/>
+      <c r="E60" s="23" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F60" s="18" t="n"/>
       <c r="G60" s="7" t="n"/>
       <c r="H60" s="7" t="n"/>
       <c r="I60" s="7" t="n"/>
@@ -2124,16 +2154,16 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>SLPTX403</t>
+          <t>고덱스</t>
         </is>
       </c>
       <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="19" t="n"/>
-      <c r="E61" s="19" t="n"/>
-      <c r="F61" s="19" t="n">
-        <v>1500</v>
-      </c>
+      <c r="D61" s="18" t="n"/>
+      <c r="E61" s="18" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F61" s="18" t="n"/>
       <c r="G61" s="7" t="n"/>
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="7" t="n"/>
@@ -2141,16 +2171,16 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>TSC프린터</t>
+          <t>라벨발행기</t>
         </is>
       </c>
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
-      <c r="D62" s="19" t="n"/>
-      <c r="E62" s="23" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F62" s="19" t="n"/>
+      <c r="D62" s="18" t="n"/>
+      <c r="E62" s="18" t="n">
+        <v>2620</v>
+      </c>
+      <c r="F62" s="18" t="n"/>
       <c r="G62" s="7" t="n"/>
       <c r="H62" s="7" t="n"/>
       <c r="I62" s="7" t="n"/>
@@ -2158,16 +2188,16 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>고덱스</t>
+          <t>라벨프린터기</t>
         </is>
       </c>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="19" t="n"/>
-      <c r="E63" s="19" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F63" s="19" t="n"/>
+      <c r="D63" s="18" t="n"/>
+      <c r="E63" s="18" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F63" s="18" t="n"/>
       <c r="G63" s="7" t="n"/>
       <c r="H63" s="7" t="n"/>
       <c r="I63" s="7" t="n"/>
@@ -2175,16 +2205,16 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>라벨발행기</t>
+          <t>라벨프린터용지</t>
         </is>
       </c>
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
-      <c r="D64" s="19" t="n"/>
-      <c r="E64" s="19" t="n">
-        <v>2620</v>
-      </c>
-      <c r="F64" s="19" t="n"/>
+      <c r="D64" s="18" t="n"/>
+      <c r="E64" s="18" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F64" s="18" t="n"/>
       <c r="G64" s="7" t="n"/>
       <c r="H64" s="7" t="n"/>
       <c r="I64" s="7" t="n"/>
@@ -2192,16 +2222,16 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>라벨프린터기</t>
+          <t>롤프린터</t>
         </is>
       </c>
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
-      <c r="D65" s="19" t="n"/>
-      <c r="E65" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F65" s="19" t="n"/>
+      <c r="D65" s="18" t="n"/>
+      <c r="E65" s="18" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F65" s="18" t="n"/>
       <c r="G65" s="7" t="n"/>
       <c r="H65" s="7" t="n"/>
       <c r="I65" s="7" t="n"/>
@@ -2209,16 +2239,16 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>라벨프린터용지</t>
+          <t>바코드구입</t>
         </is>
       </c>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
-      <c r="D66" s="19" t="n"/>
-      <c r="E66" s="19" t="n">
-        <v>2100</v>
-      </c>
-      <c r="F66" s="19" t="n"/>
+      <c r="D66" s="18" t="n"/>
+      <c r="E66" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F66" s="18" t="n"/>
       <c r="G66" s="7" t="n"/>
       <c r="H66" s="7" t="n"/>
       <c r="I66" s="7" t="n"/>
@@ -2226,16 +2256,16 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>롤프린터</t>
+          <t>바코드등록</t>
         </is>
       </c>
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="19" t="n"/>
-      <c r="E67" s="19" t="n">
-        <v>1100</v>
-      </c>
-      <c r="F67" s="19" t="n"/>
+      <c r="D67" s="18" t="n"/>
+      <c r="E67" s="18" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F67" s="18" t="n"/>
       <c r="G67" s="7" t="n"/>
       <c r="H67" s="7" t="n"/>
       <c r="I67" s="7" t="n"/>
@@ -2243,16 +2273,16 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>바코드구입</t>
+          <t>바코드라벨프린터기</t>
         </is>
       </c>
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="19" t="n"/>
-      <c r="E68" s="19" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F68" s="19" t="n"/>
+      <c r="D68" s="18" t="n"/>
+      <c r="E68" s="18" t="n">
+        <v>1700</v>
+      </c>
+      <c r="F68" s="18" t="n"/>
       <c r="G68" s="7" t="n"/>
       <c r="H68" s="7" t="n"/>
       <c r="I68" s="7" t="n"/>
@@ -2260,16 +2290,16 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>바코드등록</t>
+          <t>바코드생성</t>
         </is>
       </c>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="19" t="n"/>
-      <c r="E69" s="19" t="n">
-        <v>2200</v>
-      </c>
-      <c r="F69" s="19" t="n"/>
+      <c r="D69" s="18" t="n"/>
+      <c r="E69" s="18" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F69" s="18" t="n"/>
       <c r="G69" s="7" t="n"/>
       <c r="H69" s="7" t="n"/>
       <c r="I69" s="7" t="n"/>
@@ -2277,16 +2307,16 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>바코드라벨프린터기</t>
+          <t>바코드프린트</t>
         </is>
       </c>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
-      <c r="D70" s="19" t="n"/>
-      <c r="E70" s="19" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F70" s="19" t="n"/>
+      <c r="D70" s="18" t="n"/>
+      <c r="E70" s="18" t="n">
+        <v>1520</v>
+      </c>
+      <c r="F70" s="18" t="n"/>
       <c r="G70" s="7" t="n"/>
       <c r="H70" s="7" t="n"/>
       <c r="I70" s="7" t="n"/>
@@ -2294,16 +2324,16 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>바코드생성</t>
+          <t>산업용바코드</t>
         </is>
       </c>
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="19" t="n"/>
-      <c r="E71" s="19" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F71" s="19" t="n"/>
+      <c r="D71" s="18" t="n"/>
+      <c r="E71" s="18" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F71" s="18" t="n"/>
       <c r="G71" s="7" t="n"/>
       <c r="H71" s="7" t="n"/>
       <c r="I71" s="7" t="n"/>
@@ -2311,16 +2341,16 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>바코드프린트</t>
+          <t>소형라벨프린터</t>
         </is>
       </c>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
-      <c r="D72" s="19" t="n"/>
-      <c r="E72" s="19" t="n">
-        <v>1520</v>
-      </c>
-      <c r="F72" s="19" t="n"/>
+      <c r="D72" s="18" t="n"/>
+      <c r="E72" s="18" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F72" s="18" t="n"/>
       <c r="G72" s="7" t="n"/>
       <c r="H72" s="7" t="n"/>
       <c r="I72" s="7" t="n"/>
@@ -2328,53 +2358,19 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>산업용바코드</t>
+          <t>지브라프린터</t>
         </is>
       </c>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
-      <c r="D73" s="19" t="n"/>
-      <c r="E73" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F73" s="19" t="n"/>
+      <c r="D73" s="18" t="n"/>
+      <c r="E73" s="18" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F73" s="18" t="n"/>
       <c r="G73" s="7" t="n"/>
       <c r="H73" s="7" t="n"/>
       <c r="I73" s="7" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="6" t="inlineStr">
-        <is>
-          <t>소형라벨프린터</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="7" t="n"/>
-      <c r="D74" s="19" t="n"/>
-      <c r="E74" s="19" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F74" s="19" t="n"/>
-      <c r="G74" s="7" t="n"/>
-      <c r="H74" s="7" t="n"/>
-      <c r="I74" s="7" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>지브라프린터</t>
-        </is>
-      </c>
-      <c r="B75" s="7" t="n"/>
-      <c r="C75" s="7" t="n"/>
-      <c r="D75" s="19" t="n"/>
-      <c r="E75" s="19" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F75" s="19" t="n"/>
-      <c r="G75" s="7" t="n"/>
-      <c r="H75" s="7" t="n"/>
-      <c r="I75" s="7" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:I52"/>

</xml_diff>